<commit_message>
Replace int_member_plan_month_eligibility with fct_member_plan_month
Move member-plan-month logic into a fact model. Add days_in_month, member_month_exposure, is_dual_eligible, and receives_ltss. Move and rename the related singular tests, and add a test that a member's eligible days in a month never exceed the days in that month.
</commit_message>
<xml_diff>
--- a/docs/fact_model_curation.xlsx
+++ b/docs/fact_model_curation.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12240"/>
+    <workbookView windowWidth="12720" windowHeight="12240"/>
   </bookViews>
   <sheets>
     <sheet name="fct_member_plan_month" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="51">
   <si>
     <t>Model Definition</t>
   </si>
@@ -35,7 +35,7 @@
     <t xml:space="preserve">MODEL       </t>
   </si>
   <si>
-    <t>fct_member_plan_months</t>
+    <t>fct_member_plan_month</t>
   </si>
   <si>
     <t xml:space="preserve">GRAIN       </t>
@@ -132,9 +132,6 @@
     <t>Must be the first day of a month</t>
   </si>
   <si>
-    <t>Validate first day of month</t>
-  </si>
-  <si>
     <t>eligible_days</t>
   </si>
   <si>
@@ -163,9 +160,6 @@
   </si>
   <si>
     <t>eligible_days / days_in_month; &gt; 0 and ≤ 1; not rounded</t>
-  </si>
-  <si>
-    <t>Validate exposure range</t>
   </si>
   <si>
     <t>is_dual_eligible</t>
@@ -842,7 +836,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -851,7 +845,7 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1396,13 +1390,11 @@
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="16.6666666666667" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24.3518518518519" style="1" customWidth="1"/>
-    <col min="3" max="3" width="51.3888888888889" style="2" customWidth="1"/>
-    <col min="4" max="4" width="9.44444444444444" style="3" customWidth="1"/>
-    <col min="5" max="5" width="8.33333333333333" style="3" customWidth="1"/>
-    <col min="6" max="6" width="23.8888888888889" style="1" customWidth="1"/>
-    <col min="7" max="7" width="37.5555555555556" style="2" customWidth="1"/>
-    <col min="8" max="8" width="23.7777777777778" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.0092592592593" style="2" customWidth="1"/>
+    <col min="3" max="3" width="30.8611111111111" style="2" customWidth="1"/>
+    <col min="4" max="5" width="6.78703703703704" style="3" customWidth="1"/>
+    <col min="6" max="6" width="14.3148148148148" style="2" customWidth="1"/>
+    <col min="7" max="8" width="22.462962962963" style="2" customWidth="1"/>
     <col min="9" max="16384" width="8.88888888888889" style="1"/>
   </cols>
   <sheetData>
@@ -1412,7 +1404,7 @@
       </c>
     </row>
     <row r="2" spans="2:3">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -1420,7 +1412,7 @@
       </c>
     </row>
     <row r="3" spans="2:3">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -1428,15 +1420,15 @@
       </c>
     </row>
     <row r="4" spans="2:3">
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" ht="28.8" spans="2:4">
-      <c r="B5" s="1" t="s">
+    <row r="5" ht="43.2" spans="2:4">
+      <c r="B5" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="4" t="s">
@@ -1449,7 +1441,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="2:8">
+    <row r="9" ht="28.8" spans="2:8">
       <c r="B9" s="5" t="s">
         <v>10</v>
       </c>
@@ -1472,8 +1464,8 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="2:6">
-      <c r="B10" s="1" t="s">
+    <row r="10" ht="28.8" spans="2:6">
+      <c r="B10" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -1485,12 +1477,12 @@
       <c r="E10" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="2:6">
-      <c r="B11" s="1" t="s">
+    <row r="11" ht="28.8" spans="2:6">
+      <c r="B11" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -1502,12 +1494,12 @@
       <c r="E11" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="2:8">
-      <c r="B12" s="1" t="s">
+    <row r="12" ht="28.8" spans="2:7">
+      <c r="B12" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -1522,92 +1514,86 @@
       <c r="G12" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="H12" s="1" t="s">
+    </row>
+    <row r="13" ht="28.8" spans="2:8">
+      <c r="B13" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="13" spans="2:8">
-      <c r="B13" s="1" t="s">
+      <c r="C13" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>19</v>
       </c>
       <c r="G13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H13" s="1" t="s">
+    </row>
+    <row r="14" spans="2:7">
+      <c r="B14" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="14" spans="2:7">
-      <c r="B14" s="1" t="s">
+      <c r="C14" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>33</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>19</v>
       </c>
       <c r="G14" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" ht="28.8" spans="2:7">
+      <c r="B15" s="2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="15" ht="28.8" spans="2:8">
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>19</v>
       </c>
       <c r="G15" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" ht="28.8" spans="2:7">
+      <c r="B16" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="H15" s="1" t="s">
+      <c r="C16" s="2" t="s">
         <v>38</v>
-      </c>
-    </row>
-    <row r="16" spans="2:7">
-      <c r="B16" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>19</v>
       </c>
       <c r="G16" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" ht="28.8" spans="2:7">
+      <c r="B17" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>41</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7">
-      <c r="B17" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>43</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>19</v>
       </c>
       <c r="G17" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" ht="43.2" spans="2:5">
+      <c r="B18" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>44</v>
-      </c>
-    </row>
-    <row r="18" ht="28.8" spans="2:5">
-      <c r="B18" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>46</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>19</v>
@@ -1615,26 +1601,26 @@
     </row>
     <row r="21" spans="2:3">
       <c r="B21" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="22" ht="28.8" spans="2:3">
+      <c r="B22" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="2:3">
-      <c r="B22" s="1" t="s">
+    <row r="23" ht="43.2" spans="2:3">
+      <c r="B23" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C23" s="2" t="s">
         <v>50</v>
-      </c>
-    </row>
-    <row r="23" ht="28.8" spans="2:3">
-      <c r="B23" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add last_eligible_date to fct_member_plan_month
</commit_message>
<xml_diff>
--- a/docs/fact_model_curation.xlsx
+++ b/docs/fact_model_curation.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="12720" windowHeight="12240"/>
+    <workbookView windowWidth="28800" windowHeight="12240" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="fct_member_plan_month" sheetId="1" r:id="rId1"/>
+    <sheet name="fct_member_month" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="55">
   <si>
     <t>Model Definition</t>
   </si>
@@ -201,7 +202,41 @@
     <t>Member-month total exposure</t>
   </si>
   <si>
-    <t>Sum of member_month_exposure across plans for each member_id + month_start_date must be ≤ 1</t>
+    <t>Sum of member_month_exposure across plans for each member_id and month_start_date must be ≤ 1</t>
+  </si>
+  <si>
+    <t>fct_member_month</t>
+  </si>
+  <si>
+    <t>member_id + month_start_date</t>
+  </si>
+  <si>
+    <t>last_eligible_date</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Between </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>month_start_date</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and the last day of the month</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -825,7 +860,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -843,6 +878,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1411,12 +1449,258 @@
         <v>2</v>
       </c>
     </row>
+    <row r="3" ht="28.8" spans="2:3">
+      <c r="B3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1" spans="2:3">
+      <c r="B4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" ht="43.2" spans="2:4">
+      <c r="B5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="4"/>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" ht="28.8" spans="2:8">
+      <c r="B9" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" ht="28.8" spans="2:6">
+      <c r="B10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" ht="28.8" spans="2:6">
+      <c r="B11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" ht="28.8" spans="2:7">
+      <c r="B12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" ht="28.8" spans="2:8">
+      <c r="B13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7">
+      <c r="B14" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" ht="28.8" spans="2:7">
+      <c r="B15" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" ht="28.8" spans="2:7">
+      <c r="B16" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" ht="28.8" spans="2:7">
+      <c r="B17" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" ht="43.2" spans="2:5">
+      <c r="B18" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3">
+      <c r="B21" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="22" ht="28.8" spans="2:3">
+      <c r="B22" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="23" ht="43.2" spans="2:3">
+      <c r="B23" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
+  <cols>
+    <col min="1" max="1" width="6.41666666666667" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.0092592592593" style="2" customWidth="1"/>
+    <col min="3" max="3" width="30.8611111111111" style="2" customWidth="1"/>
+    <col min="4" max="5" width="6.78703703703704" style="3" customWidth="1"/>
+    <col min="6" max="6" width="14.3148148148148" style="2" customWidth="1"/>
+    <col min="7" max="8" width="22.462962962963" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="8.88888888888889" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="2:3">
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
     <row r="3" spans="2:3">
       <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>4</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="2:3">
@@ -1424,7 +1708,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" ht="43.2" spans="2:4">
@@ -1546,7 +1830,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" ht="28.8" spans="2:7">
+    <row r="15" ht="43.2" spans="2:7">
       <c r="B15" s="2" t="s">
         <v>34</v>
       </c>
@@ -1599,27 +1883,38 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="2:3">
-      <c r="B21" s="6" t="s">
+    <row r="19" ht="43.2" spans="2:7">
+      <c r="B19" t="s">
+        <v>53</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3">
+      <c r="B22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="22" ht="28.8" spans="2:3">
-      <c r="B22" s="2" t="s">
+    <row r="23" ht="28.8" spans="2:3">
+      <c r="B23" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C23" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="23" ht="43.2" spans="2:3">
-      <c r="B23" s="2" t="s">
+    <row r="24" ht="43.2" spans="2:3">
+      <c r="B24" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add fct_medical_claim_lines spec to fact_model_curation
Also move singular test definitions to a new singular_tests tab
</commit_message>
<xml_diff>
--- a/docs/fact_model_curation.xlsx
+++ b/docs/fact_model_curation.xlsx
@@ -4,11 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12240" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="12240" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="fct_member_plan_month" sheetId="1" r:id="rId1"/>
     <sheet name="fct_member_month" sheetId="5" r:id="rId2"/>
+    <sheet name="fct_medical_claim_lines" sheetId="7" r:id="rId3"/>
+    <sheet name="singular_tests" sheetId="8" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="292">
   <si>
     <t>Model Definition</t>
   </si>
@@ -251,6 +253,9 @@
     <t>var('analysis_through_date') — currently 2026-06-30</t>
   </si>
   <si>
+    <t>COLUMN SPECIFICATIONS</t>
+  </si>
+  <si>
     <t>data_type</t>
   </si>
   <si>
@@ -338,7 +343,7 @@
     <t>Null iff last_day(month_start_date) &gt; analysis_through_date; otherwise true iff last_eligible_date = last_day(month_start_date)</t>
   </si>
   <si>
-    <t>assert_fct_member_month_month_end_observability</t>
+    <t>assert_fct_member_month_month_end_eligibility</t>
   </si>
   <si>
     <t>month_end_plan_id</t>
@@ -416,64 +421,520 @@
     <t>Cast eligible_days, days_in_month, and plan_count to INTEGER in the final SELECT of their respective fact models for BI compatibility. Upstream INTEGER types do not necessarily carry through aggregation.</t>
   </si>
   <si>
-    <t>SINGULAR TEST</t>
-  </si>
-  <si>
-    <t>BUSINESS RULE</t>
-  </si>
-  <si>
-    <t>IMPLEMENTATION GUIDANCE</t>
-  </si>
-  <si>
-    <t>Unique member_id + month_start_date</t>
-  </si>
-  <si>
-    <t>Return duplicated member-month keys</t>
-  </si>
-  <si>
-    <t>Exposure matches upstream plan-month sum</t>
-  </si>
-  <si>
-    <t>Compare using explicit floating-point tolerance; also verify eligible days</t>
-  </si>
-  <si>
-    <t>Null iff month-end beyond cutoff; otherwise status matches last eligible date</t>
-  </si>
-  <si>
-    <t>Verify null and observed true/false cases</t>
-  </si>
-  <si>
-    <t>assert_fct_member_month_month_end_columns_populated_when_eligible</t>
-  </si>
-  <si>
-    <t>All three month-end attributes populated iff month-end eligible</t>
-  </si>
-  <si>
-    <t>Use is not true to cover false and null</t>
-  </si>
-  <si>
-    <t>assert_fct_member_month_month_end_plan_matches_source</t>
-  </si>
-  <si>
-    <t>Expected and actual month-end plan and flags match in both directions</t>
-  </si>
-  <si>
-    <t>Model: conditional aggregation selects the plan with last_eligible_date = last_day(month_start_date). Test: independently join upstream fct_member_plan_month on that date; compare with actual month_end_plan_id is not null rows using a full outer join, explicit unmatched-key checks, and is distinct from. Both sides must use matching month-end-plan filters; no-overlap ensures at most one expected plan.</t>
-  </si>
-  <si>
-    <t>GENERIC TESTS</t>
-  </si>
-  <si>
-    <t>SCOPE</t>
-  </si>
-  <si>
-    <t>NOTE</t>
-  </si>
-  <si>
-    <t>member_id, month_start_date, eligible_days, days_in_month, member_month_exposure, plan_count, has_multiple_plans, last_eligible_date</t>
-  </si>
-  <si>
-    <t>Do not require not_null on month-end status or attributes</t>
+    <t>FCT_MEDICAL_CLAIM_LINES | DESIGN CONTRACT</t>
+  </si>
+  <si>
+    <t>fct_medical_claim_lines</t>
+  </si>
+  <si>
+    <t>claim_id + claim_line_number</t>
+  </si>
+  <si>
+    <t>int_medical_claim_lines_enriched</t>
+  </si>
+  <si>
+    <t>Claim-line detail for cost and utilization analysis; preserve unmatched eligibility and all claim statuses</t>
+  </si>
+  <si>
+    <t>ATTRIBUTION</t>
+  </si>
+  <si>
+    <t>Eligibility matched using service_from_date; unmatched claims retained</t>
+  </si>
+  <si>
+    <t>NULLABILITY NOTE</t>
+  </si>
+  <si>
+    <t>Y = required non-null; N = nullable. Required claim and financial fields verified against 42,163 source rows (zero nulls).</t>
+  </si>
+  <si>
+    <t>COLUMN GROUPS</t>
+  </si>
+  <si>
+    <t>Order</t>
+  </si>
+  <si>
+    <t>Group</t>
+  </si>
+  <si>
+    <t>Columns</t>
+  </si>
+  <si>
+    <t>Claim grain</t>
+  </si>
+  <si>
+    <t>claim_id, claim_line_number</t>
+  </si>
+  <si>
+    <t>Member and eligibility</t>
+  </si>
+  <si>
+    <t>member_id, eligibility_segment_id, plan_id, has_matching_eligibility</t>
+  </si>
+  <si>
+    <t>Plan classification</t>
+  </si>
+  <si>
+    <t>state_code, product_code, aid_category_code</t>
+  </si>
+  <si>
+    <t>Claim classification</t>
+  </si>
+  <si>
+    <t>claim_type_code, claim_status_code</t>
+  </si>
+  <si>
+    <t>Service dates</t>
+  </si>
+  <si>
+    <t>service_from_date, service_to_date</t>
+  </si>
+  <si>
+    <t>Processing and audit dates</t>
+  </si>
+  <si>
+    <t>received_date, paid_date, updated_at</t>
+  </si>
+  <si>
+    <t>Financial measures</t>
+  </si>
+  <si>
+    <t>billed_amount, allowed_amount, paid_amount, member_responsibility_amount</t>
+  </si>
+  <si>
+    <t>Provider and service details</t>
+  </si>
+  <si>
+    <t>billing_provider_npi, rendering_provider_npi, billing_provider_type, bill_type_code, place_of_service_code, revenue_code, procedure_code, procedure_modifier, units</t>
+  </si>
+  <si>
+    <t>Diagnoses</t>
+  </si>
+  <si>
+    <t>diagnosis_code_1, diagnosis_code_2, diagnosis_code_3</t>
+  </si>
+  <si>
+    <t>group</t>
+  </si>
+  <si>
+    <t>business_rule / validation</t>
+  </si>
+  <si>
+    <t>claim_id</t>
+  </si>
+  <si>
+    <t>Claim identifier</t>
+  </si>
+  <si>
+    <t>Composite grain key | Test: unique combination with claim_line_number</t>
+  </si>
+  <si>
+    <t>claim_line_number</t>
+  </si>
+  <si>
+    <t>Line number within claim</t>
+  </si>
+  <si>
+    <t>Composite grain key | Test: unique combination with claim_id</t>
+  </si>
+  <si>
+    <t>Member identifier on claim</t>
+  </si>
+  <si>
+    <t>Preserve missing member identifiers; do not substitute placeholder</t>
+  </si>
+  <si>
+    <t>eligibility_segment_id</t>
+  </si>
+  <si>
+    <t>Matched eligibility segment</t>
+  </si>
+  <si>
+    <t>stg_eligibility_segments.eligibility_segment_id</t>
+  </si>
+  <si>
+    <t>Null when no eligibility match</t>
+  </si>
+  <si>
+    <t>Plan attributed through service-date eligibility</t>
+  </si>
+  <si>
+    <t>has_matching_eligibility</t>
+  </si>
+  <si>
+    <t>Whether claim matches eligibility on service_from_date</t>
+  </si>
+  <si>
+    <t>True iff matching eligibility segment exists | Test: eligibility consistency</t>
+  </si>
+  <si>
+    <t>state_code</t>
+  </si>
+  <si>
+    <t>State associated with matched plan</t>
+  </si>
+  <si>
+    <t>Null for unmatched eligibility; plan state, not member residence</t>
+  </si>
+  <si>
+    <t>product_code</t>
+  </si>
+  <si>
+    <t>Matched plan product classification</t>
+  </si>
+  <si>
+    <t>Null for unmatched eligibility</t>
+  </si>
+  <si>
+    <t>aid_category_code</t>
+  </si>
+  <si>
+    <t>Matched plan aid category</t>
+  </si>
+  <si>
+    <t>claim_type_code</t>
+  </si>
+  <si>
+    <t>Claim type classification</t>
+  </si>
+  <si>
+    <t>Preserve all claim types; verify non-null upstream</t>
+  </si>
+  <si>
+    <t>claim_status_code</t>
+  </si>
+  <si>
+    <t>Claim status classification</t>
+  </si>
+  <si>
+    <t>Retain all statuses, including denied and unpaid</t>
+  </si>
+  <si>
+    <t>service_from_date</t>
+  </si>
+  <si>
+    <t>Beginning of service period</t>
+  </si>
+  <si>
+    <t>Basis for eligibility matching | Test: service date range</t>
+  </si>
+  <si>
+    <t>service_to_date</t>
+  </si>
+  <si>
+    <t>End of service period</t>
+  </si>
+  <si>
+    <t>On or after service_from_date | Test: service date range</t>
+  </si>
+  <si>
+    <t>received_date</t>
+  </si>
+  <si>
+    <t>Date claim received for processing</t>
+  </si>
+  <si>
+    <t>May be missing before formal receipt</t>
+  </si>
+  <si>
+    <t>paid_date</t>
+  </si>
+  <si>
+    <t>Date claim paid</t>
+  </si>
+  <si>
+    <t>May be missing for unpaid or denied claims</t>
+  </si>
+  <si>
+    <t>updated_at</t>
+  </si>
+  <si>
+    <t>timestamp</t>
+  </si>
+  <si>
+    <t>Most recent source record update</t>
+  </si>
+  <si>
+    <t>Retain for traceability</t>
+  </si>
+  <si>
+    <t>billed_amount</t>
+  </si>
+  <si>
+    <t>decimal</t>
+  </si>
+  <si>
+    <t>Amount billed by provider</t>
+  </si>
+  <si>
+    <t>Preserve source amount (including negatives); no rounding or zero-fill. Required non-null; verified zero nulls / 42,163 rows.</t>
+  </si>
+  <si>
+    <t>allowed_amount</t>
+  </si>
+  <si>
+    <t>Amount recognized as allowable</t>
+  </si>
+  <si>
+    <t>paid_amount</t>
+  </si>
+  <si>
+    <t>Amount paid by payer</t>
+  </si>
+  <si>
+    <t>member_responsibility_amount</t>
+  </si>
+  <si>
+    <t>Member financial responsibility</t>
+  </si>
+  <si>
+    <t>billing_provider_npi</t>
+  </si>
+  <si>
+    <t>Billing provider NPI</t>
+  </si>
+  <si>
+    <t>Keep as text to preserve leading zeros</t>
+  </si>
+  <si>
+    <t>rendering_provider_npi</t>
+  </si>
+  <si>
+    <t>Rendering provider NPI</t>
+  </si>
+  <si>
+    <t>billing_provider_type</t>
+  </si>
+  <si>
+    <t>Billing provider classification</t>
+  </si>
+  <si>
+    <t>Preserve source value</t>
+  </si>
+  <si>
+    <t>bill_type_code</t>
+  </si>
+  <si>
+    <t>Institutional bill type classification</t>
+  </si>
+  <si>
+    <t>May be absent for noninstitutional claims</t>
+  </si>
+  <si>
+    <t>place_of_service_code</t>
+  </si>
+  <si>
+    <t>Service setting code</t>
+  </si>
+  <si>
+    <t>revenue_code</t>
+  </si>
+  <si>
+    <t>Institutional revenue code</t>
+  </si>
+  <si>
+    <t>procedure_code</t>
+  </si>
+  <si>
+    <t>Procedure or service code</t>
+  </si>
+  <si>
+    <t>procedure_modifier</t>
+  </si>
+  <si>
+    <t>Procedure modifier</t>
+  </si>
+  <si>
+    <t>Optional service detail</t>
+  </si>
+  <si>
+    <t>units</t>
+  </si>
+  <si>
+    <t>numeric</t>
+  </si>
+  <si>
+    <t>Units of service</t>
+  </si>
+  <si>
+    <t>Preserve negatives for adjustments and nulls for missing values</t>
+  </si>
+  <si>
+    <t>diagnosis_code_1</t>
+  </si>
+  <si>
+    <t>First recorded diagnosis</t>
+  </si>
+  <si>
+    <t>Preserve missing values and source code</t>
+  </si>
+  <si>
+    <t>diagnosis_code_2</t>
+  </si>
+  <si>
+    <t>Second recorded diagnosis</t>
+  </si>
+  <si>
+    <t>diagnosis_code_3</t>
+  </si>
+  <si>
+    <t>Third recorded diagnosis</t>
+  </si>
+  <si>
+    <t>SINGULAR TESTS | GOLD FACT MODELS</t>
+  </si>
+  <si>
+    <t>test_filename</t>
+  </si>
+  <si>
+    <t>validation_objective</t>
+  </si>
+  <si>
+    <t>reference_model</t>
+  </si>
+  <si>
+    <t>validation_logic</t>
+  </si>
+  <si>
+    <t>failure_condition</t>
+  </si>
+  <si>
+    <t>implementation_notes</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>assert_fct_member_month_unique_grain.sql</t>
+  </si>
+  <si>
+    <t>One row per member and month</t>
+  </si>
+  <si>
+    <t>Group by member_id, month_start_date</t>
+  </si>
+  <si>
+    <t>Any key with count &gt; 1</t>
+  </si>
+  <si>
+    <t>Existing singular test; member_id and month_start_date are grain keys.</t>
+  </si>
+  <si>
+    <t>Passing</t>
+  </si>
+  <si>
+    <t>assert_fct_member_month_exposure_reconciles.sql</t>
+  </si>
+  <si>
+    <t>Reconcile eligible days and member-month exposure</t>
+  </si>
+  <si>
+    <t>fct_member_plan_month ↔ fct_member_month</t>
+  </si>
+  <si>
+    <t>Aggregate plan-month records by member_id + month_start_date; compare eligible_days and member_month_exposure</t>
+  </si>
+  <si>
+    <t>Any unmatched or unequal eligible days or exposure beyond tolerance</t>
+  </si>
+  <si>
+    <t>Use explicit floating-point tolerance; test against upstream independent aggregation.</t>
+  </si>
+  <si>
+    <t>assert_fct_member_month_month_end_eligibility.sql</t>
+  </si>
+  <si>
+    <t>Validate month-end eligibility and analysis cutoff</t>
+  </si>
+  <si>
+    <t>Compare calendar month-end to analysis_through_date and last_eligible_date</t>
+  </si>
+  <si>
+    <t>Unexpected null or incorrect month-end eligibility status</t>
+  </si>
+  <si>
+    <t>Month-end eligibility must be null when calendar month-end is beyond cutoff.</t>
+  </si>
+  <si>
+    <t>assert_fct_member_month_month_end_columns_populated_when_eligible.sql</t>
+  </si>
+  <si>
+    <t>Check month-end attributes are populated only when eligible</t>
+  </si>
+  <si>
+    <t>Validate month_end_plan_id, is_dual_eligible_month_end and receives_ltss_month_end relative to is_eligible_month_end</t>
+  </si>
+  <si>
+    <t>Missing values for eligible month-end or values populated otherwise</t>
+  </si>
+  <si>
+    <t>Use IS NOT TRUE to cover both false and null.</t>
+  </si>
+  <si>
+    <t>assert_fct_member_month_month_end_plan_matches_source.sql</t>
+  </si>
+  <si>
+    <t>Independently validate month-end plan and classification</t>
+  </si>
+  <si>
+    <t>Find month-end plan in upstream plan-month fact and compare plan and flags</t>
+  </si>
+  <si>
+    <t>Missing, extra, or mismatched month-end plan/flags</t>
+  </si>
+  <si>
+    <t>Compare independently derived expected month-end plan and flags in both directions.</t>
+  </si>
+  <si>
+    <t>assert_fct_medical_claim_lines_unique_grain.sql</t>
+  </si>
+  <si>
+    <t>One fact row per claim_id + claim_line_number</t>
+  </si>
+  <si>
+    <t>Group by claim_id, claim_line_number</t>
+  </si>
+  <si>
+    <t>Any key combination with count &gt; 1</t>
+  </si>
+  <si>
+    <t>Return duplicate keys; not_null grain keys covered by generic tests.</t>
+  </si>
+  <si>
+    <t>Planned</t>
+  </si>
+  <si>
+    <t>assert_fct_medical_claim_lines_source_reconciliation.sql</t>
+  </si>
+  <si>
+    <t>Every intermediate claim line appears exactly once in fact</t>
+  </si>
+  <si>
+    <t>int_medical_claim_lines_enriched ↔ fct_medical_claim_lines</t>
+  </si>
+  <si>
+    <t>Compare composite key sets in both directions (full outer join or EXCEPT)</t>
+  </si>
+  <si>
+    <t>Any missing or extra claim-line key</t>
+  </si>
+  <si>
+    <t>Row counts alone are insufficient; retain all claim statuses and unmatched-eligibility lines.</t>
+  </si>
+  <si>
+    <t>assert_fct_medical_claim_lines_financial_reconciliation.sql</t>
+  </si>
+  <si>
+    <t>Verify four financial amounts remain unchanged</t>
+  </si>
+  <si>
+    <t>Join by claim_id + claim_line_number and compare four measures with null-safe equality</t>
+  </si>
+  <si>
+    <t>Any billed, allowed, paid or member-responsibility amount differs</t>
+  </si>
+  <si>
+    <t>Exact comparison; no rounding or zero-fill; negative amounts remain valid.</t>
   </si>
 </sst>
 </file>
@@ -486,7 +947,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -494,22 +955,78 @@
       <charset val="134"/>
     </font>
     <font>
+      <b/>
+      <sz val="15"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF17324B"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="11"/>
-      <name val="Carlito"/>
+      <color rgb="FF183153"/>
+      <name val="Calibri"/>
       <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Carlito"/>
+      <name val="Calibri"/>
       <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <name val="Carlito"/>
+      <color rgb="FF16324F"/>
+      <name val="Calibri"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -592,13 +1109,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
@@ -628,20 +1138,31 @@
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="35">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF19344D"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCE8F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3F7FA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -651,7 +1172,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAF3F5"/>
+        <fgColor rgb="FF16324F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCE8F1"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -968,76 +1495,64 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1046,10 +1561,10 @@
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1058,10 +1573,10 @@
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1070,10 +1585,10 @@
     <xf numFmtId="0" fontId="0" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1082,10 +1597,10 @@
     <xf numFmtId="0" fontId="0" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1094,48 +1609,111 @@
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1611,252 +2189,252 @@
   <dimension ref="A1:H23"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="16.6666666666667" style="8" customWidth="1"/>
-    <col min="2" max="2" width="19.0092592592593" style="9" customWidth="1"/>
-    <col min="3" max="3" width="52.8333333333333" style="9" customWidth="1"/>
-    <col min="4" max="5" width="9.37037037037037" style="10" customWidth="1"/>
-    <col min="6" max="6" width="24.0648148148148" style="9" customWidth="1"/>
-    <col min="7" max="7" width="41.962962962963" style="9" customWidth="1"/>
-    <col min="8" max="8" width="25.5462962962963" style="9" customWidth="1"/>
-    <col min="9" max="16384" width="8.88888888888889" style="8"/>
+    <col min="1" max="1" width="16.6666666666667" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.0092592592593" style="26" customWidth="1"/>
+    <col min="3" max="3" width="52.8333333333333" style="26" customWidth="1"/>
+    <col min="4" max="5" width="9.37037037037037" style="27" customWidth="1"/>
+    <col min="6" max="6" width="24.0648148148148" style="26" customWidth="1"/>
+    <col min="7" max="7" width="41.962962962963" style="26" customWidth="1"/>
+    <col min="8" max="8" width="25.5462962962963" style="26" customWidth="1"/>
+    <col min="9" max="16384" width="8.88888888888889" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="2:3">
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="26" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="2:3">
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="26" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="2:3">
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="26" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" ht="28.8" spans="2:4">
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="9"/>
+      <c r="D5" s="26"/>
     </row>
     <row r="8" spans="1:1">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="2:8">
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="H9" s="28" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" spans="2:6">
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="26" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="11" spans="2:6">
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="26" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="12" spans="2:7">
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="26" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="13" spans="2:8">
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="H13" s="26" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="14" spans="2:7">
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E14" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="26" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="15" ht="28.8" spans="2:7">
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="26" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="16" spans="2:7">
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="E16" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="26" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="17" spans="2:7">
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="E17" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="26" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="18" ht="28.8" spans="2:5">
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E18" s="27" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="19" ht="43.2" spans="2:7">
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="10" t="s">
+      <c r="E19" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="G19" s="26" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="21" spans="2:3">
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="26" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="22" spans="2:3">
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" s="26" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="23" ht="28.8" spans="2:3">
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="26" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1869,22 +2447,1553 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H39"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="13.8" outlineLevelCol="7"/>
+  <dimension ref="A1:H31"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="33.1111111111111" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24.4444444444444" style="1" customWidth="1"/>
-    <col min="3" max="3" width="45.2222222222222" style="1" customWidth="1"/>
-    <col min="4" max="5" width="5.88888888888889" style="1" customWidth="1"/>
-    <col min="6" max="6" width="16.2222222222222" style="1" customWidth="1"/>
-    <col min="7" max="7" width="49.4444444444444" style="1" customWidth="1"/>
-    <col min="8" max="8" width="69.3333333333333" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="10" style="1"/>
+    <col min="1" max="1" width="33.1111111111111" style="19" customWidth="1"/>
+    <col min="2" max="2" width="24.4444444444444" style="19" customWidth="1"/>
+    <col min="3" max="3" width="45.2222222222222" style="19" customWidth="1"/>
+    <col min="4" max="5" width="5.88888888888889" style="19" customWidth="1"/>
+    <col min="6" max="6" width="16.2222222222222" style="19" customWidth="1"/>
+    <col min="7" max="7" width="49.4444444444444" style="19" customWidth="1"/>
+    <col min="8" max="8" width="69.3333333333333" style="19" customWidth="1"/>
+    <col min="9" max="16384" width="10" style="19"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" s="18" customFormat="1" ht="18" spans="1:8">
+      <c r="A1" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" customFormat="1" ht="18" spans="1:8">
+      <c r="A8" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+    </row>
+    <row r="9" s="19" customFormat="1" ht="28.8" spans="1:8">
+      <c r="A9" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="H9" s="13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" ht="28.8" spans="1:8">
+      <c r="A10" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="H10" s="22" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="D11" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="22"/>
+      <c r="G11" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="H11" s="22" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="H12" s="22" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" s="22"/>
+      <c r="G13" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="H13" s="22"/>
+    </row>
+    <row r="14" ht="28" customHeight="1" spans="1:8">
+      <c r="A14" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" s="22"/>
+      <c r="G14" s="22" t="s">
+        <v>80</v>
+      </c>
+      <c r="H14" s="22" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="22" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22" t="s">
+        <v>83</v>
+      </c>
+      <c r="H15" s="22"/>
+    </row>
+    <row r="16" ht="28.8" spans="1:8">
+      <c r="A16" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="H16" s="22"/>
+    </row>
+    <row r="17" ht="26" customHeight="1" spans="1:8">
+      <c r="A17" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>88</v>
+      </c>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="F17" s="22"/>
+      <c r="G17" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="H17" s="22"/>
+    </row>
+    <row r="18" ht="43.2" spans="1:8">
+      <c r="A18" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="H18" s="22" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1" spans="1:8">
+      <c r="A19" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="F19" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="G19" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="H19" s="22" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="20" ht="28.8" spans="1:8">
+      <c r="A20" s="22" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>100</v>
+      </c>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="H20" s="22" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="21" ht="28.8" spans="1:8">
+      <c r="A21" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>103</v>
+      </c>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="F21" s="22"/>
+      <c r="G21" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="H21" s="22" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="23" s="18" customFormat="1" ht="19" customHeight="1" spans="1:8">
+      <c r="A23" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="B23" s="23" t="s">
+        <v>105</v>
+      </c>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23"/>
+      <c r="H23" s="23"/>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" s="22" t="s">
+        <v>106</v>
+      </c>
+      <c r="B24" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="24"/>
+      <c r="H24" s="24"/>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" s="22" t="s">
+        <v>108</v>
+      </c>
+      <c r="B25" s="24" t="s">
+        <v>109</v>
+      </c>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="24"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="24"/>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="B26" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="24"/>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="B27" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="24"/>
+    </row>
+    <row r="28" spans="1:8">
+      <c r="A28" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="B28" s="24" t="s">
+        <v>115</v>
+      </c>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="24"/>
+    </row>
+    <row r="29" spans="1:8">
+      <c r="A29" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="B29" s="24" t="s">
+        <v>117</v>
+      </c>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="24"/>
+      <c r="G29" s="24"/>
+      <c r="H29" s="24"/>
+    </row>
+    <row r="30" spans="1:8">
+      <c r="A30" s="25" t="s">
+        <v>118</v>
+      </c>
+      <c r="B30" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="24"/>
+      <c r="H30" s="24"/>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="25"/>
+      <c r="B31" s="25"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="B24:H24"/>
+    <mergeCell ref="B25:H25"/>
+    <mergeCell ref="B26:H26"/>
+    <mergeCell ref="B27:H27"/>
+    <mergeCell ref="B28:H28"/>
+    <mergeCell ref="B29:H29"/>
+    <mergeCell ref="B30:H30"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:H54"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
+  <cols>
+    <col min="1" max="1" width="23.7777777777778" style="6" customWidth="1"/>
+    <col min="2" max="2" width="28.2222222222222" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11.2222222222222" style="1" customWidth="1"/>
+    <col min="4" max="4" width="39" style="1" customWidth="1"/>
+    <col min="5" max="6" width="9.88888888888889" style="1" customWidth="1"/>
+    <col min="7" max="7" width="29" style="1" customWidth="1"/>
+    <col min="8" max="8" width="80" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88888888888889" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="29" customHeight="1" spans="1:8">
+      <c r="A1" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" ht="25" customHeight="1" spans="1:8">
+      <c r="A9" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="14">
+        <v>1</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="14">
+        <v>2</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="14">
+        <v>3</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="14">
+        <v>4</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="14">
+        <v>5</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="14">
+        <v>6</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" s="14">
+        <v>7</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" s="14">
+        <v>8</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="14">
+        <v>9</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="14"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+    </row>
+    <row r="21" ht="25" customHeight="1" spans="1:8">
+      <c r="A21" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" s="16"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H22" s="13" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G26" s="17" t="s">
+        <v>163</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="28" ht="28.8" spans="1:8">
+      <c r="A28" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
+      <c r="A29" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
+      <c r="A30" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G30" s="4"/>
+      <c r="H30" s="4" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
+      <c r="A31" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G31" s="4"/>
+      <c r="H31" s="4" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G35" s="4"/>
+      <c r="H35" s="4" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G36" s="4"/>
+      <c r="H36" s="4" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G37" s="4"/>
+      <c r="H37" s="4" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G38" s="4"/>
+      <c r="H38" s="4" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="39" ht="28.8" spans="1:8">
+      <c r="A39" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="40" ht="28.8" spans="1:8">
+      <c r="A40" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G40" s="4"/>
+      <c r="H40" s="4" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="41" ht="28.8" spans="1:8">
+      <c r="A41" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G41" s="4"/>
+      <c r="H41" s="4" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="42" ht="28.8" spans="1:8">
+      <c r="A42" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G42" s="4"/>
+      <c r="H42" s="4" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G43" s="4"/>
+      <c r="H43" s="4" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G44" s="4"/>
+      <c r="H44" s="4" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G45" s="4"/>
+      <c r="H45" s="4" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="A46" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G46" s="4"/>
+      <c r="H46" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="A47" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G47" s="4"/>
+      <c r="H47" s="4" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
+      <c r="A48" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G48" s="4"/>
+      <c r="H48" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="E49" s="4"/>
+      <c r="F49" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G49" s="4"/>
+      <c r="H49" s="4" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G50" s="4"/>
+      <c r="H50" s="4" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G51" s="4"/>
+      <c r="H51" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
+      <c r="A52" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="E52" s="4"/>
+      <c r="F52" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G52" s="4"/>
+      <c r="H52" s="4" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
+      <c r="A53" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="E53" s="4"/>
+      <c r="F53" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G53" s="4"/>
+      <c r="H53" s="4" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
+      <c r="A54" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="E54" s="4"/>
+      <c r="F54" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G54" s="4"/>
+      <c r="H54" s="4" t="s">
+        <v>235</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="C11:H11"/>
+    <mergeCell ref="C12:H12"/>
+    <mergeCell ref="C13:H13"/>
+    <mergeCell ref="C14:H14"/>
+    <mergeCell ref="C15:H15"/>
+    <mergeCell ref="C16:H16"/>
+    <mergeCell ref="C17:H17"/>
+    <mergeCell ref="C18:H18"/>
+    <mergeCell ref="C19:H19"/>
+    <mergeCell ref="A21:B21"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="6"/>
+  <cols>
+    <col min="1" max="1" width="52.3333333333333" style="1" customWidth="1"/>
+    <col min="2" max="2" width="34.8888888888889" style="1" customWidth="1"/>
+    <col min="3" max="3" width="29.5555555555556" style="1" customWidth="1"/>
+    <col min="4" max="4" width="52.4444444444444" style="1" customWidth="1"/>
+    <col min="5" max="6" width="40" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="9" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1" spans="1:7">
       <c r="A1" s="2" t="s">
-        <v>54</v>
+        <v>240</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1892,512 +4001,217 @@
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-    </row>
-    <row r="2" spans="1:2">
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B2" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="3" ht="28.8" spans="1:7">
+      <c r="A3" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="8" ht="27.6" spans="1:8">
-      <c r="A8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" ht="27.6" spans="1:8">
-      <c r="A9" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
+      <c r="D3" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="4" ht="43.2" spans="1:7">
+      <c r="A4" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="5" ht="28.8" spans="1:7">
+      <c r="A5" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="6" ht="28.8" spans="1:7">
+      <c r="A6" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="7" ht="28.8" spans="1:7">
+      <c r="A7" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="8" ht="28.8" spans="1:7">
+      <c r="A8" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="9" ht="28.8" spans="1:7">
+      <c r="A9" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="10" ht="28.8" spans="1:7">
       <c r="A10" s="5" t="s">
-        <v>24</v>
+        <v>287</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>69</v>
+        <v>288</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>70</v>
+        <v>283</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>19</v>
+        <v>289</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" s="5"/>
+        <v>290</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>291</v>
+      </c>
       <c r="G10" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="H12" s="5"/>
-    </row>
-    <row r="13" ht="28" customHeight="1" spans="1:8">
-      <c r="A13" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="H14" s="5"/>
-    </row>
-    <row r="15" ht="27.6" spans="1:8">
-      <c r="A15" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="H15" s="5"/>
-    </row>
-    <row r="16" ht="26" customHeight="1" spans="1:8">
-      <c r="A16" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="H16" s="5"/>
-    </row>
-    <row r="17" ht="41.4" spans="1:8">
-      <c r="A17" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="18" ht="40" customHeight="1" spans="1:8">
-      <c r="A18" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="H18" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="19" ht="27.6" spans="1:8">
-      <c r="A19" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="H19" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="20" ht="27.6" spans="1:8">
-      <c r="A20" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="C22" s="6"/>
-    </row>
-    <row r="23" ht="30" customHeight="1" spans="1:3">
-      <c r="A23" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="C23" s="7"/>
-    </row>
-    <row r="24" ht="41" customHeight="1" spans="1:3">
-      <c r="A24" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="C24" s="7"/>
-    </row>
-    <row r="25" ht="30" customHeight="1" spans="1:3">
-      <c r="A25" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="C25" s="7"/>
-    </row>
-    <row r="26" ht="44" customHeight="1" spans="1:3">
-      <c r="A26" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="B26" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="C26" s="7"/>
-    </row>
-    <row r="27" ht="44" customHeight="1" spans="1:3">
-      <c r="A27" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="C27" s="7"/>
-    </row>
-    <row r="28" ht="32" customHeight="1" spans="1:3">
-      <c r="A28" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="C28" s="7"/>
-    </row>
-    <row r="29" ht="49" customHeight="1" spans="1:3">
-      <c r="A29" t="s">
-        <v>117</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="C29" s="7"/>
-    </row>
-    <row r="30" ht="14.4" spans="1:2">
-      <c r="A30"/>
-      <c r="B30"/>
-    </row>
-    <row r="31" ht="27" customHeight="1" spans="1:3">
-      <c r="A31" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="32" ht="33" customHeight="1" spans="1:3">
-      <c r="A32" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="33" ht="32" customHeight="1" spans="1:3">
-      <c r="A33" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="34" ht="43" customHeight="1" spans="1:3">
-      <c r="A34" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="35" ht="46" customHeight="1" spans="1:3">
-      <c r="A35" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="36" ht="72" customHeight="1" spans="1:3">
-      <c r="A36" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="38" ht="27" customHeight="1" spans="1:3">
-      <c r="A38" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="39" ht="55" customHeight="1" spans="1:3">
-      <c r="A39" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B39" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="C39" s="5" t="s">
-        <v>138</v>
+        <v>280</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Add fct_medical_claim_lines model with generic tests
</commit_message>
<xml_diff>
--- a/docs/fact_model_curation.xlsx
+++ b/docs/fact_model_curation.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12240" activeTab="2"/>
+    <workbookView windowWidth="28800" windowHeight="12240" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="fct_member_plan_month" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="310">
   <si>
     <t>Model Definition</t>
   </si>
@@ -439,7 +439,8 @@
     <t>ATTRIBUTION</t>
   </si>
   <si>
-    <t>Eligibility matched using service_from_date; unmatched claims retained</t>
+    <t>Eligibility matched using service_from_date; unmatched claims retained
+All 42,163 source claim lines have service_from_date on or before analysis_through_date (2026-06-30). Preserve all claim lines in the fact model. Apply the analysis cutoff in downstream PMPM calculations to align claim costs with member exposure.</t>
   </si>
   <si>
     <t>NULLABILITY NOTE</t>
@@ -619,6 +620,18 @@
     <t>Basis for eligibility matching | Test: service date range</t>
   </si>
   <si>
+    <t>service_from_month_start_date</t>
+  </si>
+  <si>
+    <t>First calendar day of the month containing service_from_date; used to attribute claim lines to a reporting month for monthly claims aggregation and PMPM analysis.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Derived as the first calendar day of the month containing service_from_date; must equal date_trunc('month', service_from_date).</t>
+  </si>
+  <si>
     <t>service_to_date</t>
   </si>
   <si>
@@ -805,6 +818,12 @@
     <t>Status</t>
   </si>
   <si>
+    <t>priority</t>
+  </si>
+  <si>
+    <t>model_name</t>
+  </si>
+  <si>
     <t>assert_fct_member_month_unique_grain.sql</t>
   </si>
   <si>
@@ -823,6 +842,9 @@
     <t>Passing</t>
   </si>
   <si>
+    <t>High</t>
+  </si>
+  <si>
     <t>assert_fct_member_month_exposure_reconciles.sql</t>
   </si>
   <si>
@@ -935,6 +957,39 @@
   </si>
   <si>
     <t>Exact comparison; no rounding or zero-fill; negative amounts remain valid.</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>assert_fct_medical_claim_lines_eligibility_consistency.sql</t>
+  </si>
+  <si>
+    <t>Verify eligibility-match flag agrees with populated identifiers</t>
+  </si>
+  <si>
+    <t>Matched: flag true and both eligibility_segment_id and plan_id present; unmatched: flag false and both identifiers null</t>
+  </si>
+  <si>
+    <t>Any null flag or disagreement between flag and identifiers</t>
+  </si>
+  <si>
+    <t>Check both matched and unmatched rows; use IS TRUE / IS FALSE to catch null flags.</t>
+  </si>
+  <si>
+    <t>assert_fct_medical_claim_lines_service_date_range.sql</t>
+  </si>
+  <si>
+    <t>Ensure service period dates are chronological</t>
+  </si>
+  <si>
+    <t>Compare service_to_date &gt;= service_from_date for each claim line</t>
+  </si>
+  <si>
+    <t>Any service_to_date earlier than service_from_date</t>
+  </si>
+  <si>
+    <t>Equal start and end dates are valid; not_null checks are maintained in YAML.</t>
   </si>
 </sst>
 </file>
@@ -947,7 +1002,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1005,28 +1060,11 @@
       <sz val="14"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -1138,8 +1176,15 @@
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="39">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1155,12 +1200,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDCE8F0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF3F7FA"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1495,144 +1534,147 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1641,31 +1683,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1674,46 +1722,43 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2189,252 +2234,252 @@
   <dimension ref="A1:H23"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="16.6666666666667" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.0092592592593" style="26" customWidth="1"/>
-    <col min="3" max="3" width="52.8333333333333" style="26" customWidth="1"/>
-    <col min="4" max="5" width="9.37037037037037" style="27" customWidth="1"/>
-    <col min="6" max="6" width="24.0648148148148" style="26" customWidth="1"/>
-    <col min="7" max="7" width="41.962962962963" style="26" customWidth="1"/>
-    <col min="8" max="8" width="25.5462962962963" style="26" customWidth="1"/>
-    <col min="9" max="16384" width="8.88888888888889" style="1"/>
+    <col min="1" max="1" width="16.6666666666667" style="2" customWidth="1"/>
+    <col min="2" max="2" width="19.0092592592593" style="21" customWidth="1"/>
+    <col min="3" max="3" width="52.8333333333333" style="21" customWidth="1"/>
+    <col min="4" max="5" width="9.37037037037037" style="12" customWidth="1"/>
+    <col min="6" max="6" width="24.0648148148148" style="21" customWidth="1"/>
+    <col min="7" max="7" width="41.962962962963" style="21" customWidth="1"/>
+    <col min="8" max="8" width="25.5462962962963" style="21" customWidth="1"/>
+    <col min="9" max="16384" width="8.88888888888889" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="2:3">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="C2" s="21" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="2:3">
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="26" t="s">
+      <c r="C3" s="21" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="2:3">
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="C4" s="21" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" ht="28.8" spans="2:4">
-      <c r="B5" s="26" t="s">
+      <c r="B5" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="26" t="s">
+      <c r="C5" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="26"/>
+      <c r="D5" s="21"/>
     </row>
     <row r="8" spans="1:1">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="2:8">
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="28" t="s">
+      <c r="D9" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="28" t="s">
+      <c r="E9" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="28" t="s">
+      <c r="F9" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="28" t="s">
+      <c r="G9" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="28" t="s">
+      <c r="H9" s="29" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" spans="2:6">
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="26" t="s">
+      <c r="C10" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="27" t="s">
+      <c r="E10" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="26" t="s">
+      <c r="F10" s="21" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="11" spans="2:6">
-      <c r="B11" s="26" t="s">
+      <c r="B11" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="26" t="s">
+      <c r="C11" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="27" t="s">
+      <c r="D11" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="27" t="s">
+      <c r="E11" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="26" t="s">
+      <c r="F11" s="21" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="12" spans="2:7">
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="26" t="s">
+      <c r="C12" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="27" t="s">
+      <c r="D12" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="27" t="s">
+      <c r="E12" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G12" s="26" t="s">
+      <c r="G12" s="21" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="13" spans="2:8">
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="26" t="s">
+      <c r="C13" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="E13" s="27" t="s">
+      <c r="E13" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G13" s="26" t="s">
+      <c r="G13" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="H13" s="26" t="s">
+      <c r="H13" s="21" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="14" spans="2:7">
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="26" t="s">
+      <c r="C14" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="27" t="s">
+      <c r="E14" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G14" s="26" t="s">
+      <c r="G14" s="21" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="15" ht="28.8" spans="2:7">
-      <c r="B15" s="26" t="s">
+      <c r="B15" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="26" t="s">
+      <c r="C15" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="E15" s="27" t="s">
+      <c r="E15" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G15" s="26" t="s">
+      <c r="G15" s="21" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="16" spans="2:7">
-      <c r="B16" s="26" t="s">
+      <c r="B16" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="26" t="s">
+      <c r="C16" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="E16" s="27" t="s">
+      <c r="E16" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G16" s="26" t="s">
+      <c r="G16" s="21" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="17" spans="2:7">
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="26" t="s">
+      <c r="C17" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="E17" s="27" t="s">
+      <c r="E17" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G17" s="26" t="s">
+      <c r="G17" s="21" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="18" ht="28.8" spans="2:5">
-      <c r="B18" s="26" t="s">
+      <c r="B18" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="26" t="s">
+      <c r="C18" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="27" t="s">
+      <c r="E18" s="12" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="19" ht="43.2" spans="2:7">
-      <c r="B19" s="26" t="s">
+      <c r="B19" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="26" t="s">
+      <c r="C19" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="27" t="s">
+      <c r="E19" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G19" s="26" t="s">
+      <c r="G19" s="21" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="21" spans="2:3">
-      <c r="B21" s="29" t="s">
+      <c r="B21" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="26" t="s">
+      <c r="C21" s="21" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="22" spans="2:3">
-      <c r="B22" s="26" t="s">
+      <c r="B22" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="C22" s="26" t="s">
+      <c r="C22" s="21" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="23" ht="28.8" spans="2:3">
-      <c r="B23" s="26" t="s">
+      <c r="B23" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="26" t="s">
+      <c r="C23" s="21" t="s">
         <v>53</v>
       </c>
     </row>
@@ -2450,485 +2495,485 @@
   <dimension ref="A1:H31"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="33.1111111111111" style="19" customWidth="1"/>
-    <col min="2" max="2" width="24.4444444444444" style="19" customWidth="1"/>
-    <col min="3" max="3" width="45.2222222222222" style="19" customWidth="1"/>
-    <col min="4" max="5" width="5.88888888888889" style="19" customWidth="1"/>
-    <col min="6" max="6" width="16.2222222222222" style="19" customWidth="1"/>
-    <col min="7" max="7" width="49.4444444444444" style="19" customWidth="1"/>
-    <col min="8" max="8" width="69.3333333333333" style="19" customWidth="1"/>
-    <col min="9" max="16384" width="10" style="19"/>
+    <col min="1" max="1" width="33.1111111111111" style="23" customWidth="1"/>
+    <col min="2" max="2" width="24.4444444444444" style="23" customWidth="1"/>
+    <col min="3" max="3" width="45.2222222222222" style="23" customWidth="1"/>
+    <col min="4" max="5" width="5.88888888888889" style="23" customWidth="1"/>
+    <col min="6" max="6" width="16.2222222222222" style="23" customWidth="1"/>
+    <col min="7" max="7" width="49.4444444444444" style="23" customWidth="1"/>
+    <col min="8" max="8" width="69.3333333333333" style="23" customWidth="1"/>
+    <col min="9" max="16384" width="10" style="23"/>
   </cols>
   <sheetData>
-    <row r="1" s="18" customFormat="1" ht="18" spans="1:8">
-      <c r="A1" s="20" t="s">
+    <row r="1" s="22" customFormat="1" ht="18" spans="1:8">
+      <c r="A1" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="23" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="23" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="23" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="23" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="23" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="8" customFormat="1" ht="18" spans="1:8">
-      <c r="A8" s="16" t="s">
+    <row r="8" ht="18" spans="1:8">
+      <c r="A8" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-    </row>
-    <row r="9" s="19" customFormat="1" ht="28.8" spans="1:8">
-      <c r="A9" s="12" t="s">
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+    </row>
+    <row r="9" s="23" customFormat="1" ht="28.8" spans="1:8">
+      <c r="A9" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="G9" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="H9" s="16" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" ht="28.8" spans="1:8">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="22" t="s">
+      <c r="C10" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="22" t="s">
+      <c r="F10" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="G10" s="22" t="s">
+      <c r="G10" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="H10" s="22" t="s">
+      <c r="H10" s="25" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="C11" s="25" t="s">
         <v>71</v>
       </c>
-      <c r="D11" s="22" t="s">
+      <c r="D11" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="22" t="s">
+      <c r="E11" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="22"/>
-      <c r="G11" s="22" t="s">
+      <c r="F11" s="25"/>
+      <c r="G11" s="25" t="s">
         <v>71</v>
       </c>
-      <c r="H11" s="22" t="s">
+      <c r="H11" s="25" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="22" t="s">
+      <c r="A12" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22" t="s">
+      <c r="D12" s="25"/>
+      <c r="E12" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="22"/>
-      <c r="G12" s="22" t="s">
+      <c r="F12" s="25"/>
+      <c r="G12" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="H12" s="22" t="s">
+      <c r="H12" s="25" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="C13" s="22" t="s">
+      <c r="C13" s="25" t="s">
         <v>76</v>
       </c>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22" t="s">
+      <c r="D13" s="25"/>
+      <c r="E13" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="22"/>
-      <c r="G13" s="22" t="s">
+      <c r="F13" s="25"/>
+      <c r="G13" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="H13" s="22"/>
+      <c r="H13" s="25"/>
     </row>
     <row r="14" ht="28" customHeight="1" spans="1:8">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="C14" s="22" t="s">
+      <c r="C14" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22" t="s">
+      <c r="D14" s="25"/>
+      <c r="E14" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="F14" s="22"/>
-      <c r="G14" s="22" t="s">
+      <c r="F14" s="25"/>
+      <c r="G14" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="H14" s="22" t="s">
+      <c r="H14" s="25" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="C15" s="22" t="s">
+      <c r="C15" s="25" t="s">
         <v>82</v>
       </c>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22" t="s">
+      <c r="D15" s="25"/>
+      <c r="E15" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22" t="s">
+      <c r="F15" s="25"/>
+      <c r="G15" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="22"/>
+      <c r="H15" s="25"/>
     </row>
     <row r="16" ht="28.8" spans="1:8">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22" t="s">
+      <c r="D16" s="25"/>
+      <c r="E16" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="F16" s="22"/>
-      <c r="G16" s="22" t="s">
+      <c r="F16" s="25"/>
+      <c r="G16" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="H16" s="22"/>
+      <c r="H16" s="25"/>
     </row>
     <row r="17" ht="26" customHeight="1" spans="1:8">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="22" t="s">
+      <c r="B17" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22" t="s">
+      <c r="D17" s="25"/>
+      <c r="E17" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="F17" s="22"/>
-      <c r="G17" s="22" t="s">
+      <c r="F17" s="25"/>
+      <c r="G17" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="H17" s="22"/>
+      <c r="H17" s="25"/>
     </row>
     <row r="18" ht="43.2" spans="1:8">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="C18" s="22" t="s">
+      <c r="C18" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22" t="s">
+      <c r="D18" s="25"/>
+      <c r="E18" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22" t="s">
+      <c r="F18" s="25"/>
+      <c r="G18" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="H18" s="22" t="s">
+      <c r="H18" s="25" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="19" ht="40" customHeight="1" spans="1:8">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="B19" s="22" t="s">
+      <c r="B19" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="C19" s="22" t="s">
+      <c r="C19" s="25" t="s">
         <v>96</v>
       </c>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22" t="s">
+      <c r="D19" s="25"/>
+      <c r="E19" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="F19" s="22" t="s">
+      <c r="F19" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="G19" s="22" t="s">
+      <c r="G19" s="25" t="s">
         <v>97</v>
       </c>
-      <c r="H19" s="22" t="s">
+      <c r="H19" s="25" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="20" ht="28.8" spans="1:8">
-      <c r="A20" s="22" t="s">
+      <c r="A20" s="25" t="s">
         <v>99</v>
       </c>
-      <c r="B20" s="22" t="s">
+      <c r="B20" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="C20" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22" t="s">
+      <c r="D20" s="25"/>
+      <c r="E20" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22" t="s">
+      <c r="F20" s="25"/>
+      <c r="G20" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="H20" s="22" t="s">
+      <c r="H20" s="25" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="21" ht="28.8" spans="1:8">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="25" t="s">
         <v>102</v>
       </c>
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="C21" s="22" t="s">
+      <c r="C21" s="25" t="s">
         <v>103</v>
       </c>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22" t="s">
+      <c r="D21" s="25"/>
+      <c r="E21" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="F21" s="22"/>
-      <c r="G21" s="22" t="s">
+      <c r="F21" s="25"/>
+      <c r="G21" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="H21" s="22" t="s">
+      <c r="H21" s="25" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="23" s="18" customFormat="1" ht="19" customHeight="1" spans="1:8">
-      <c r="A23" s="20" t="s">
+    <row r="23" s="22" customFormat="1" ht="19" customHeight="1" spans="1:8">
+      <c r="A23" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="B23" s="23" t="s">
+      <c r="B23" s="26" t="s">
         <v>105</v>
       </c>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="23"/>
-      <c r="G23" s="23"/>
-      <c r="H23" s="23"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="25" t="s">
         <v>106</v>
       </c>
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="27" t="s">
         <v>107</v>
       </c>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="24"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="25" t="s">
         <v>108</v>
       </c>
-      <c r="B25" s="24" t="s">
+      <c r="B25" s="27" t="s">
         <v>109</v>
       </c>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
-      <c r="G25" s="24"/>
-      <c r="H25" s="24"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="27"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="22" t="s">
+      <c r="A26" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="B26" s="24" t="s">
+      <c r="B26" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="24"/>
-      <c r="H26" s="24"/>
+      <c r="C26" s="27"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="27"/>
+      <c r="H26" s="27"/>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="B27" s="24" t="s">
+      <c r="B27" s="27" t="s">
         <v>113</v>
       </c>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
-      <c r="G27" s="24"/>
-      <c r="H27" s="24"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="27"/>
     </row>
     <row r="28" spans="1:8">
-      <c r="A28" s="22" t="s">
+      <c r="A28" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="B28" s="24" t="s">
+      <c r="B28" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
-      <c r="G28" s="24"/>
-      <c r="H28" s="24"/>
+      <c r="C28" s="27"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="27"/>
+      <c r="F28" s="27"/>
+      <c r="G28" s="27"/>
+      <c r="H28" s="27"/>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="22" t="s">
+      <c r="A29" s="25" t="s">
         <v>116</v>
       </c>
-      <c r="B29" s="24" t="s">
+      <c r="B29" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="24"/>
-      <c r="H29" s="24"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="27"/>
+      <c r="G29" s="27"/>
+      <c r="H29" s="27"/>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="25" t="s">
+      <c r="A30" s="28" t="s">
         <v>118</v>
       </c>
-      <c r="B30" s="24" t="s">
+      <c r="B30" s="27" t="s">
         <v>119</v>
       </c>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="24"/>
-      <c r="F30" s="24"/>
-      <c r="G30" s="24"/>
-      <c r="H30" s="24"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="27"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="27"/>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="25"/>
-      <c r="B31" s="25"/>
+      <c r="A31" s="28"/>
+      <c r="B31" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -2950,1016 +2995,1082 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="23.7777777777778" style="6" customWidth="1"/>
-    <col min="2" max="2" width="28.2222222222222" style="1" customWidth="1"/>
-    <col min="3" max="3" width="11.2222222222222" style="1" customWidth="1"/>
-    <col min="4" max="4" width="39" style="1" customWidth="1"/>
-    <col min="5" max="6" width="9.88888888888889" style="1" customWidth="1"/>
-    <col min="7" max="7" width="29" style="1" customWidth="1"/>
-    <col min="8" max="8" width="80" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.88888888888889" style="1"/>
+    <col min="1" max="1" width="23.7777777777778" style="8" customWidth="1"/>
+    <col min="2" max="2" width="28.2222222222222" style="2" customWidth="1"/>
+    <col min="3" max="3" width="11.2222222222222" style="2" customWidth="1"/>
+    <col min="4" max="4" width="39" style="2" customWidth="1"/>
+    <col min="5" max="6" width="9.88888888888889" style="2" customWidth="1"/>
+    <col min="7" max="7" width="29" style="2" customWidth="1"/>
+    <col min="8" max="8" width="80" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="8.88888888888889" style="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="29" customHeight="1" spans="1:8">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="9" t="s">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="9" t="s">
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="9" t="s">
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="8" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="9" t="s">
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="8" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="9" t="s">
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+    </row>
+    <row r="6" ht="31" customHeight="1" spans="1:8">
+      <c r="A6" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="12" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="9" t="s">
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="8" t="s">
         <v>128</v>
       </c>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
     </row>
     <row r="9" ht="25" customHeight="1" spans="1:8">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="16" t="s">
         <v>132</v>
       </c>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="14">
+      <c r="A11" s="17">
         <v>1</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="14">
+      <c r="A12" s="17">
         <v>2</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="14">
+      <c r="A13" s="17">
         <v>3</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="14">
+      <c r="A14" s="17">
         <v>4</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="C14" s="15" t="s">
+      <c r="C14" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="14">
+      <c r="A15" s="17">
         <v>5</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="18" t="s">
         <v>142</v>
       </c>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="14">
+      <c r="A16" s="17">
         <v>6</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="18" t="s">
         <v>144</v>
       </c>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="18"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="14">
+      <c r="A17" s="17">
         <v>7</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="C17" s="15" t="s">
+      <c r="C17" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="14">
+      <c r="A18" s="17">
         <v>8</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C18" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
     </row>
     <row r="19" spans="1:8">
-      <c r="A19" s="14">
+      <c r="A19" s="17">
         <v>9</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C19" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="14"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
+      <c r="A20" s="17"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
     </row>
     <row r="21" ht="25" customHeight="1" spans="1:8">
-      <c r="A21" s="16" t="s">
+      <c r="A21" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="B21" s="16"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="14"/>
     </row>
     <row r="22" spans="1:8">
-      <c r="A22" s="12" t="s">
+      <c r="A22" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="D22" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="E22" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="F22" s="13" t="s">
+      <c r="F22" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="G22" s="13" t="s">
+      <c r="G22" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H22" s="13" t="s">
+      <c r="H22" s="16" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="23" spans="1:8">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="17" t="s">
         <v>133</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="F23" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4" t="s">
+      <c r="G23" s="5"/>
+      <c r="H23" s="5" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="17" t="s">
         <v>133</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4" t="s">
+      <c r="G24" s="5"/>
+      <c r="H24" s="5" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4" t="s">
+      <c r="E25" s="5"/>
+      <c r="F25" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="G25" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H25" s="4" t="s">
+      <c r="H25" s="5" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="14" t="s">
+      <c r="A26" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4" t="s">
+      <c r="E26" s="5"/>
+      <c r="F26" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G26" s="17" t="s">
+      <c r="G26" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="H26" s="4" t="s">
+      <c r="H26" s="5" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="14" t="s">
+      <c r="A27" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4" t="s">
+      <c r="E27" s="5"/>
+      <c r="F27" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="G27" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H27" s="4" t="s">
+      <c r="H27" s="5" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="28" ht="28.8" spans="1:8">
-      <c r="A28" s="14" t="s">
+      <c r="A28" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4" t="s">
+      <c r="E28" s="5"/>
+      <c r="F28" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4" t="s">
+      <c r="G28" s="5"/>
+      <c r="H28" s="5" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="14" t="s">
+      <c r="A29" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4" t="s">
+      <c r="E29" s="5"/>
+      <c r="F29" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4" t="s">
+      <c r="G29" s="5"/>
+      <c r="H29" s="5" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="14" t="s">
+      <c r="A30" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4" t="s">
+      <c r="E30" s="5"/>
+      <c r="F30" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G30" s="4"/>
-      <c r="H30" s="4" t="s">
+      <c r="G30" s="5"/>
+      <c r="H30" s="5" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="31" spans="1:8">
-      <c r="A31" s="14" t="s">
+      <c r="A31" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="D31" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4" t="s">
+      <c r="E31" s="5"/>
+      <c r="F31" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G31" s="4"/>
-      <c r="H31" s="4" t="s">
+      <c r="G31" s="5"/>
+      <c r="H31" s="5" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="32" spans="1:8">
-      <c r="A32" s="14" t="s">
+      <c r="A32" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C32" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="D32" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4" t="s">
+      <c r="E32" s="5"/>
+      <c r="F32" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G32" s="4"/>
-      <c r="H32" s="4" t="s">
+      <c r="G32" s="5"/>
+      <c r="H32" s="5" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="33" spans="1:8">
-      <c r="A33" s="14" t="s">
+      <c r="A33" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="D33" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4" t="s">
+      <c r="E33" s="5"/>
+      <c r="F33" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4" t="s">
+      <c r="G33" s="5"/>
+      <c r="H33" s="5" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="34" spans="1:8">
-      <c r="A34" s="14" t="s">
+      <c r="A34" s="17" t="s">
         <v>141</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="D34" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4" t="s">
+      <c r="E34" s="5"/>
+      <c r="F34" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4" t="s">
+      <c r="G34" s="5"/>
+      <c r="H34" s="5" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="35" spans="1:8">
-      <c r="A35" s="14" t="s">
+    <row r="35" ht="60" customHeight="1" spans="1:8">
+      <c r="A35" s="17" t="s">
         <v>141</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D35" s="4" t="s">
+      <c r="D35" s="21" t="s">
         <v>187</v>
       </c>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4" t="s">
+      <c r="E35" s="31" t="s">
+        <v>188</v>
+      </c>
+      <c r="F35" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4" t="s">
-        <v>188</v>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="36" spans="1:8">
-      <c r="A36" s="14" t="s">
+      <c r="A36" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37" s="17" t="s">
         <v>143</v>
       </c>
-      <c r="B36" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="C36" s="4" t="s">
+      <c r="B37" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="C37" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D36" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4" t="s">
+      <c r="D37" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G36" s="4"/>
-      <c r="H36" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8">
-      <c r="A37" s="14" t="s">
+      <c r="G37" s="5"/>
+      <c r="H37" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" s="17" t="s">
         <v>143</v>
       </c>
-      <c r="B37" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="C37" s="4" t="s">
+      <c r="B38" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="C38" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D37" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4" t="s">
+      <c r="D38" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8">
-      <c r="A38" s="14" t="s">
+      <c r="G38" s="5"/>
+      <c r="H38" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" s="17" t="s">
         <v>143</v>
       </c>
-      <c r="B38" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="E38" s="4"/>
-      <c r="F38" s="4" t="s">
+      <c r="B39" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="E39" s="5"/>
+      <c r="F39" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G38" s="4"/>
-      <c r="H38" s="4" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="39" ht="28.8" spans="1:8">
-      <c r="A39" s="14" t="s">
+      <c r="G39" s="5"/>
+      <c r="H39" s="5" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="40" ht="28.8" spans="1:8">
+      <c r="A40" s="17" t="s">
         <v>145</v>
       </c>
-      <c r="B39" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4" t="s">
+      <c r="B40" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="40" ht="28.8" spans="1:8">
-      <c r="A40" s="14" t="s">
+      <c r="G40" s="5"/>
+      <c r="H40" s="5" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="41" ht="28.8" spans="1:8">
+      <c r="A41" s="17" t="s">
         <v>145</v>
       </c>
-      <c r="B40" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="D40" s="4" t="s">
+      <c r="B41" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="C41" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="E40" s="4"/>
-      <c r="F40" s="4" t="s">
+      <c r="D41" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G40" s="4"/>
-      <c r="H40" s="4" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="41" ht="28.8" spans="1:8">
-      <c r="A41" s="14" t="s">
+      <c r="G41" s="5"/>
+      <c r="H41" s="5" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="42" ht="28.8" spans="1:8">
+      <c r="A42" s="17" t="s">
         <v>145</v>
       </c>
-      <c r="B41" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="D41" s="4" t="s">
+      <c r="B42" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G42" s="5"/>
+      <c r="H42" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="E41" s="4"/>
-      <c r="F41" s="4" t="s">
+    </row>
+    <row r="43" ht="28.8" spans="1:8">
+      <c r="A43" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="E43" s="5"/>
+      <c r="F43" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G41" s="4"/>
-      <c r="H41" s="4" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="42" ht="28.8" spans="1:8">
-      <c r="A42" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="D42" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="E42" s="4"/>
-      <c r="F42" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="G42" s="4"/>
-      <c r="H42" s="4" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8">
-      <c r="A43" s="14" t="s">
+      <c r="G43" s="5"/>
+      <c r="H43" s="5" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="B43" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="C43" s="4" t="s">
+      <c r="B44" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="C44" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D43" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="E43" s="4"/>
-      <c r="F43" s="4" t="s">
+      <c r="D44" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G43" s="4"/>
-      <c r="H43" s="4" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8">
-      <c r="A44" s="14" t="s">
+      <c r="G44" s="5"/>
+      <c r="H44" s="5" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="B44" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="C44" s="4" t="s">
+      <c r="B45" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="C45" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D44" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="E44" s="4"/>
-      <c r="F44" s="4" t="s">
+      <c r="D45" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8">
-      <c r="A45" s="14" t="s">
+      <c r="G45" s="5"/>
+      <c r="H45" s="5" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="A46" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="B45" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="C45" s="4" t="s">
+      <c r="B46" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="C46" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D45" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4" t="s">
+      <c r="D46" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="E46" s="5"/>
+      <c r="F46" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8">
-      <c r="A46" s="14" t="s">
+      <c r="G46" s="5"/>
+      <c r="H46" s="5" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="A47" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="B46" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="C46" s="4" t="s">
+      <c r="B47" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="C47" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D46" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="E46" s="4"/>
-      <c r="F46" s="4" t="s">
+      <c r="D47" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="E47" s="5"/>
+      <c r="F47" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G46" s="4"/>
-      <c r="H46" s="4" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8">
-      <c r="A47" s="14" t="s">
+      <c r="G47" s="5"/>
+      <c r="H47" s="5" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
+      <c r="A48" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="B48" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="E48" s="5"/>
+      <c r="F48" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="C47" s="4" t="s">
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="C49" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D47" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="E47" s="4"/>
-      <c r="F47" s="4" t="s">
+      <c r="D49" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G47" s="4"/>
-      <c r="H47" s="4" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8">
-      <c r="A48" s="14" t="s">
+      <c r="G49" s="5"/>
+      <c r="H49" s="5" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="B48" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="C48" s="4" t="s">
+      <c r="B50" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="C50" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D48" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="E48" s="4"/>
-      <c r="F48" s="4" t="s">
+      <c r="D50" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="E50" s="5"/>
+      <c r="F50" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8">
-      <c r="A49" s="14" t="s">
+      <c r="G50" s="5"/>
+      <c r="H50" s="5" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="B49" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="C49" s="4" t="s">
+      <c r="B51" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="C51" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D49" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="E49" s="4"/>
-      <c r="F49" s="4" t="s">
+      <c r="D51" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G49" s="4"/>
-      <c r="H49" s="4" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8">
-      <c r="A50" s="14" t="s">
+      <c r="G51" s="5"/>
+      <c r="H51" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
+      <c r="A52" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="B50" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="C50" s="4" t="s">
+      <c r="B52" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="E52" s="5"/>
+      <c r="F52" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
+      <c r="A53" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="B53" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="C53" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D50" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="E50" s="4"/>
-      <c r="F50" s="4" t="s">
+      <c r="D53" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="E53" s="5"/>
+      <c r="F53" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G50" s="4"/>
-      <c r="H50" s="4" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8">
-      <c r="A51" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="C51" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="E51" s="4"/>
-      <c r="F51" s="4" t="s">
+      <c r="G53" s="5"/>
+      <c r="H53" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
+      <c r="A54" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="E54" s="5"/>
+      <c r="F54" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G51" s="4"/>
-      <c r="H51" s="4" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8">
-      <c r="A52" s="14" t="s">
+      <c r="G54" s="5"/>
+      <c r="H54" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
+      <c r="A55" s="17" t="s">
         <v>149</v>
       </c>
-      <c r="B52" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="C52" s="4" t="s">
+      <c r="B55" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="C55" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D52" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="E52" s="4"/>
-      <c r="F52" s="4" t="s">
+      <c r="D55" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="E55" s="5"/>
+      <c r="F55" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G52" s="4"/>
-      <c r="H52" s="4" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8">
-      <c r="A53" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D53" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="E53" s="4"/>
-      <c r="F53" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="G53" s="4"/>
-      <c r="H53" s="4" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8">
-      <c r="A54" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="C54" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D54" s="4" t="s">
+      <c r="G55" s="5"/>
+      <c r="H55" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="E54" s="4"/>
-      <c r="F54" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="G54" s="4"/>
-      <c r="H54" s="4" t="s">
-        <v>235</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="17">
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B7:H7"/>
     <mergeCell ref="C11:H11"/>
     <mergeCell ref="C12:H12"/>
     <mergeCell ref="C13:H13"/>
@@ -3979,240 +4090,353 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="6"/>
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="52.3333333333333" style="1" customWidth="1"/>
-    <col min="2" max="2" width="34.8888888888889" style="1" customWidth="1"/>
-    <col min="3" max="3" width="29.5555555555556" style="1" customWidth="1"/>
-    <col min="4" max="4" width="52.4444444444444" style="1" customWidth="1"/>
-    <col min="5" max="6" width="40" style="1" customWidth="1"/>
-    <col min="7" max="7" width="8" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="9" style="1"/>
+    <col min="1" max="1" width="49.1111111111111" style="2" customWidth="1"/>
+    <col min="2" max="2" width="34.8888888888889" style="2" customWidth="1"/>
+    <col min="3" max="3" width="29" style="2" customWidth="1"/>
+    <col min="4" max="4" width="52.4444444444444" style="2" customWidth="1"/>
+    <col min="5" max="6" width="40" style="2" customWidth="1"/>
+    <col min="7" max="7" width="8" style="2" customWidth="1"/>
+    <col min="8" max="8" width="7.44444444444444" style="2" customWidth="1"/>
+    <col min="9" max="9" width="21.5555555555556" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1" spans="1:7">
-      <c r="A1" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="D2" s="3" t="s">
+    <row r="1" ht="25" customHeight="1" spans="1:9">
+      <c r="A1" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+    </row>
+    <row r="2" ht="27" customHeight="1" spans="1:9">
+      <c r="A2" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="3" ht="28.8" spans="1:7">
-      <c r="A3" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="F2" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="3" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A3" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>250</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>251</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>252</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="4" ht="43.2" spans="1:7">
+      <c r="D3" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
       <c r="A4" s="5" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="F4" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="G4" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="G4" s="5" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="5" ht="28.8" spans="1:7">
-      <c r="A5" s="4" t="s">
+      <c r="H4" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="I4" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>263</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="6" ht="28.8" spans="1:7">
+    </row>
+    <row r="5" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A5" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
       <c r="A6" s="5" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>56</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="7" ht="28.8" spans="1:7">
-      <c r="A7" s="4" t="s">
-        <v>270</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>273</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="8" ht="28.8" spans="1:7">
+        <v>259</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A7" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
       <c r="A8" s="5" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>121</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="9" ht="28.8" spans="1:7">
-      <c r="A9" s="4" t="s">
-        <v>281</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>282</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>285</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>286</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="10" ht="28.8" spans="1:7">
+        <v>287</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="9" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A9" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
       <c r="A10" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="G10" s="5" t="s">
         <v>287</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>288</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>283</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>289</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>290</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>291</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>280</v>
+      <c r="H10" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="11" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A11" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="12" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A12" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
Add singular tests for fct_medical_claim_lines
</commit_message>
<xml_diff>
--- a/docs/fact_model_curation.xlsx
+++ b/docs/fact_model_curation.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="309">
   <si>
     <t>Model Definition</t>
   </si>
@@ -921,9 +921,6 @@
   </si>
   <si>
     <t>Return duplicate keys; not_null grain keys covered by generic tests.</t>
-  </si>
-  <si>
-    <t>Planned</t>
   </si>
   <si>
     <t>assert_fct_medical_claim_lines_source_reconciliation.sql</t>
@@ -1184,7 +1181,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="40">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1200,6 +1197,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDCE8F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.05"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.05"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1408,12 +1417,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.25"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.25"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.25"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.25"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1540,7 +1564,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1552,119 +1576,119 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1677,52 +1701,64 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1743,7 +1779,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2235,12 +2271,12 @@
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="16.6666666666667" style="2" customWidth="1"/>
-    <col min="2" max="2" width="19.0092592592593" style="21" customWidth="1"/>
-    <col min="3" max="3" width="52.8333333333333" style="21" customWidth="1"/>
-    <col min="4" max="5" width="9.37037037037037" style="12" customWidth="1"/>
-    <col min="6" max="6" width="24.0648148148148" style="21" customWidth="1"/>
-    <col min="7" max="7" width="41.962962962963" style="21" customWidth="1"/>
-    <col min="8" max="8" width="25.5462962962963" style="21" customWidth="1"/>
+    <col min="2" max="2" width="19.0092592592593" style="25" customWidth="1"/>
+    <col min="3" max="3" width="52.8333333333333" style="25" customWidth="1"/>
+    <col min="4" max="5" width="9.37037037037037" style="15" customWidth="1"/>
+    <col min="6" max="6" width="24.0648148148148" style="25" customWidth="1"/>
+    <col min="7" max="7" width="41.962962962963" style="25" customWidth="1"/>
+    <col min="8" max="8" width="25.5462962962963" style="25" customWidth="1"/>
     <col min="9" max="16384" width="8.88888888888889" style="2"/>
   </cols>
   <sheetData>
@@ -2250,37 +2286,37 @@
       </c>
     </row>
     <row r="2" spans="2:3">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="25" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="2:3">
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="25" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="2:3">
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="25" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" ht="28.8" spans="2:4">
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="21"/>
+      <c r="D5" s="25"/>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="2" t="s">
@@ -2288,198 +2324,198 @@
       </c>
     </row>
     <row r="9" spans="2:8">
-      <c r="B9" s="29" t="s">
+      <c r="B9" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="29" t="s">
+      <c r="D9" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="29" t="s">
+      <c r="E9" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="29" t="s">
+      <c r="F9" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="29" t="s">
+      <c r="G9" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="29" t="s">
+      <c r="H9" s="33" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" spans="2:6">
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="21" t="s">
+      <c r="F10" s="25" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="11" spans="2:6">
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="21" t="s">
+      <c r="F11" s="25" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="12" spans="2:7">
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="C12" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="E12" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="G12" s="21" t="s">
+      <c r="G12" s="25" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="13" spans="2:8">
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="21" t="s">
+      <c r="C13" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="E13" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="G13" s="21" t="s">
+      <c r="G13" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="H13" s="21" t="s">
+      <c r="H13" s="25" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="14" spans="2:7">
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="C14" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="12" t="s">
+      <c r="E14" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="G14" s="21" t="s">
+      <c r="G14" s="25" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="15" ht="28.8" spans="2:7">
-      <c r="B15" s="21" t="s">
+      <c r="B15" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="C15" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="E15" s="12" t="s">
+      <c r="E15" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="G15" s="21" t="s">
+      <c r="G15" s="25" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="16" spans="2:7">
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C16" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="E16" s="12" t="s">
+      <c r="E16" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="G16" s="21" t="s">
+      <c r="G16" s="25" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="17" spans="2:7">
-      <c r="B17" s="21" t="s">
+      <c r="B17" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="C17" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="E17" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="G17" s="21" t="s">
+      <c r="G17" s="25" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="18" ht="28.8" spans="2:5">
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="E18" s="15" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="19" ht="43.2" spans="2:7">
-      <c r="B19" s="21" t="s">
+      <c r="B19" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="21" t="s">
+      <c r="C19" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="12" t="s">
+      <c r="E19" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="G19" s="21" t="s">
+      <c r="G19" s="25" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="21" spans="2:3">
-      <c r="B21" s="30" t="s">
+      <c r="B21" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="21" t="s">
+      <c r="C21" s="25" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="22" spans="2:3">
-      <c r="B22" s="21" t="s">
+      <c r="B22" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="C22" s="21" t="s">
+      <c r="C22" s="25" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="23" ht="28.8" spans="2:3">
-      <c r="B23" s="21" t="s">
+      <c r="B23" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="21" t="s">
+      <c r="C23" s="25" t="s">
         <v>53</v>
       </c>
     </row>
@@ -2495,485 +2531,485 @@
   <dimension ref="A1:H31"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="33.1111111111111" style="23" customWidth="1"/>
-    <col min="2" max="2" width="24.4444444444444" style="23" customWidth="1"/>
-    <col min="3" max="3" width="45.2222222222222" style="23" customWidth="1"/>
-    <col min="4" max="5" width="5.88888888888889" style="23" customWidth="1"/>
-    <col min="6" max="6" width="16.2222222222222" style="23" customWidth="1"/>
-    <col min="7" max="7" width="49.4444444444444" style="23" customWidth="1"/>
-    <col min="8" max="8" width="69.3333333333333" style="23" customWidth="1"/>
-    <col min="9" max="16384" width="10" style="23"/>
+    <col min="1" max="1" width="33.1111111111111" style="27" customWidth="1"/>
+    <col min="2" max="2" width="24.4444444444444" style="27" customWidth="1"/>
+    <col min="3" max="3" width="45.2222222222222" style="27" customWidth="1"/>
+    <col min="4" max="5" width="5.88888888888889" style="27" customWidth="1"/>
+    <col min="6" max="6" width="16.2222222222222" style="27" customWidth="1"/>
+    <col min="7" max="7" width="49.4444444444444" style="27" customWidth="1"/>
+    <col min="8" max="8" width="69.3333333333333" style="27" customWidth="1"/>
+    <col min="9" max="16384" width="10" style="27"/>
   </cols>
   <sheetData>
-    <row r="1" s="22" customFormat="1" ht="18" spans="1:8">
-      <c r="A1" s="10" t="s">
+    <row r="1" s="26" customFormat="1" ht="18" spans="1:8">
+      <c r="A1" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="27" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="27" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="24" t="s">
+      <c r="A4" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="27" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="27" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="27" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="8" ht="18" spans="1:8">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="B8" s="19"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-      <c r="F8" s="19"/>
-      <c r="G8" s="19"/>
-      <c r="H8" s="19"/>
-    </row>
-    <row r="9" s="23" customFormat="1" ht="28.8" spans="1:8">
-      <c r="A9" s="15" t="s">
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+    </row>
+    <row r="9" s="27" customFormat="1" ht="28.8" spans="1:8">
+      <c r="A9" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="F9" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="16" t="s">
+      <c r="G9" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="H9" s="19" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" ht="28.8" spans="1:8">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="29" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="25" t="s">
+      <c r="D10" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="25" t="s">
+      <c r="F10" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="G10" s="25" t="s">
+      <c r="G10" s="29" t="s">
         <v>68</v>
       </c>
-      <c r="H10" s="25" t="s">
+      <c r="H10" s="29" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="29" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="D11" s="25" t="s">
+      <c r="D11" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="25" t="s">
+      <c r="E11" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25" t="s">
+      <c r="F11" s="29"/>
+      <c r="G11" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="H11" s="25" t="s">
+      <c r="H11" s="29" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="25" t="s">
+      <c r="A12" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="29" t="s">
         <v>73</v>
       </c>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25" t="s">
+      <c r="D12" s="29"/>
+      <c r="E12" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25" t="s">
+      <c r="F12" s="29"/>
+      <c r="G12" s="29" t="s">
         <v>74</v>
       </c>
-      <c r="H12" s="25" t="s">
+      <c r="H12" s="29" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="25" t="s">
+      <c r="A13" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="C13" s="25" t="s">
+      <c r="C13" s="29" t="s">
         <v>76</v>
       </c>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25" t="s">
+      <c r="D13" s="29"/>
+      <c r="E13" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25" t="s">
+      <c r="F13" s="29"/>
+      <c r="G13" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="H13" s="25"/>
+      <c r="H13" s="29"/>
     </row>
     <row r="14" ht="28" customHeight="1" spans="1:8">
-      <c r="A14" s="25" t="s">
+      <c r="A14" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="C14" s="29" t="s">
         <v>79</v>
       </c>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25" t="s">
+      <c r="D14" s="29"/>
+      <c r="E14" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25" t="s">
+      <c r="F14" s="29"/>
+      <c r="G14" s="29" t="s">
         <v>80</v>
       </c>
-      <c r="H14" s="25" t="s">
+      <c r="H14" s="29" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="25" t="s">
+      <c r="A15" s="29" t="s">
         <v>81</v>
       </c>
-      <c r="B15" s="25" t="s">
+      <c r="B15" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="29" t="s">
         <v>82</v>
       </c>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25" t="s">
+      <c r="D15" s="29"/>
+      <c r="E15" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25" t="s">
+      <c r="F15" s="29"/>
+      <c r="G15" s="29" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="25"/>
+      <c r="H15" s="29"/>
     </row>
     <row r="16" ht="28.8" spans="1:8">
-      <c r="A16" s="25" t="s">
+      <c r="A16" s="29" t="s">
         <v>84</v>
       </c>
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="C16" s="25" t="s">
+      <c r="C16" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25" t="s">
+      <c r="D16" s="29"/>
+      <c r="E16" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25" t="s">
+      <c r="F16" s="29"/>
+      <c r="G16" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="H16" s="25"/>
+      <c r="H16" s="29"/>
     </row>
     <row r="17" ht="26" customHeight="1" spans="1:8">
-      <c r="A17" s="25" t="s">
+      <c r="A17" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="25" t="s">
+      <c r="B17" s="29" t="s">
         <v>70</v>
       </c>
-      <c r="C17" s="25" t="s">
+      <c r="C17" s="29" t="s">
         <v>88</v>
       </c>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25" t="s">
+      <c r="D17" s="29"/>
+      <c r="E17" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25" t="s">
+      <c r="F17" s="29"/>
+      <c r="G17" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="H17" s="25"/>
+      <c r="H17" s="29"/>
     </row>
     <row r="18" ht="43.2" spans="1:8">
-      <c r="A18" s="25" t="s">
+      <c r="A18" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="B18" s="25" t="s">
+      <c r="B18" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="C18" s="25" t="s">
+      <c r="C18" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25" t="s">
+      <c r="D18" s="29"/>
+      <c r="E18" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25" t="s">
+      <c r="F18" s="29"/>
+      <c r="G18" s="29" t="s">
         <v>93</v>
       </c>
-      <c r="H18" s="25" t="s">
+      <c r="H18" s="29" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="19" ht="40" customHeight="1" spans="1:8">
-      <c r="A19" s="25" t="s">
+      <c r="A19" s="29" t="s">
         <v>95</v>
       </c>
-      <c r="B19" s="25" t="s">
+      <c r="B19" s="29" t="s">
         <v>67</v>
       </c>
-      <c r="C19" s="25" t="s">
+      <c r="C19" s="29" t="s">
         <v>96</v>
       </c>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25" t="s">
+      <c r="D19" s="29"/>
+      <c r="E19" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="F19" s="25" t="s">
+      <c r="F19" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="G19" s="25" t="s">
+      <c r="G19" s="29" t="s">
         <v>97</v>
       </c>
-      <c r="H19" s="25" t="s">
+      <c r="H19" s="29" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="20" ht="28.8" spans="1:8">
-      <c r="A20" s="25" t="s">
+      <c r="A20" s="29" t="s">
         <v>99</v>
       </c>
-      <c r="B20" s="25" t="s">
+      <c r="B20" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="C20" s="25" t="s">
+      <c r="C20" s="29" t="s">
         <v>100</v>
       </c>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25" t="s">
+      <c r="D20" s="29"/>
+      <c r="E20" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25" t="s">
+      <c r="F20" s="29"/>
+      <c r="G20" s="29" t="s">
         <v>101</v>
       </c>
-      <c r="H20" s="25" t="s">
+      <c r="H20" s="29" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="21" ht="28.8" spans="1:8">
-      <c r="A21" s="25" t="s">
+      <c r="A21" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="B21" s="25" t="s">
+      <c r="B21" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="C21" s="25" t="s">
+      <c r="C21" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25" t="s">
+      <c r="D21" s="29"/>
+      <c r="E21" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25" t="s">
+      <c r="F21" s="29"/>
+      <c r="G21" s="29" t="s">
         <v>101</v>
       </c>
-      <c r="H21" s="25" t="s">
+      <c r="H21" s="29" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="23" s="22" customFormat="1" ht="19" customHeight="1" spans="1:8">
-      <c r="A23" s="10" t="s">
+    <row r="23" s="26" customFormat="1" ht="19" customHeight="1" spans="1:8">
+      <c r="A23" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="B23" s="26" t="s">
+      <c r="B23" s="30" t="s">
         <v>105</v>
       </c>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="26"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="30"/>
+      <c r="G23" s="30"/>
+      <c r="H23" s="30"/>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="25" t="s">
+      <c r="A24" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="B24" s="27" t="s">
+      <c r="B24" s="31" t="s">
         <v>107</v>
       </c>
-      <c r="C24" s="27"/>
-      <c r="D24" s="27"/>
-      <c r="E24" s="27"/>
-      <c r="F24" s="27"/>
-      <c r="G24" s="27"/>
-      <c r="H24" s="27"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="31"/>
+      <c r="G24" s="31"/>
+      <c r="H24" s="31"/>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="25" t="s">
+      <c r="A25" s="29" t="s">
         <v>108</v>
       </c>
-      <c r="B25" s="27" t="s">
+      <c r="B25" s="31" t="s">
         <v>109</v>
       </c>
-      <c r="C25" s="27"/>
-      <c r="D25" s="27"/>
-      <c r="E25" s="27"/>
-      <c r="F25" s="27"/>
-      <c r="G25" s="27"/>
-      <c r="H25" s="27"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="31"/>
+      <c r="F25" s="31"/>
+      <c r="G25" s="31"/>
+      <c r="H25" s="31"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="25" t="s">
+      <c r="A26" s="29" t="s">
         <v>110</v>
       </c>
-      <c r="B26" s="27" t="s">
+      <c r="B26" s="31" t="s">
         <v>111</v>
       </c>
-      <c r="C26" s="27"/>
-      <c r="D26" s="27"/>
-      <c r="E26" s="27"/>
-      <c r="F26" s="27"/>
-      <c r="G26" s="27"/>
-      <c r="H26" s="27"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="25" t="s">
+      <c r="A27" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B27" s="27" t="s">
+      <c r="B27" s="31" t="s">
         <v>113</v>
       </c>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="27"/>
-      <c r="F27" s="27"/>
-      <c r="G27" s="27"/>
-      <c r="H27" s="27"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="31"/>
+      <c r="G27" s="31"/>
+      <c r="H27" s="31"/>
     </row>
     <row r="28" spans="1:8">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="29" t="s">
         <v>114</v>
       </c>
-      <c r="B28" s="27" t="s">
+      <c r="B28" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="C28" s="27"/>
-      <c r="D28" s="27"/>
-      <c r="E28" s="27"/>
-      <c r="F28" s="27"/>
-      <c r="G28" s="27"/>
-      <c r="H28" s="27"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="31"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="31"/>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="25" t="s">
+      <c r="A29" s="29" t="s">
         <v>116</v>
       </c>
-      <c r="B29" s="27" t="s">
+      <c r="B29" s="31" t="s">
         <v>117</v>
       </c>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="27"/>
-      <c r="F29" s="27"/>
-      <c r="G29" s="27"/>
-      <c r="H29" s="27"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="31"/>
+      <c r="G29" s="31"/>
+      <c r="H29" s="31"/>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="28" t="s">
+      <c r="A30" s="32" t="s">
         <v>118</v>
       </c>
-      <c r="B30" s="27" t="s">
+      <c r="B30" s="31" t="s">
         <v>119</v>
       </c>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="27"/>
+      <c r="C30" s="31"/>
+      <c r="D30" s="31"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="31"/>
+      <c r="G30" s="31"/>
+      <c r="H30" s="31"/>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="28"/>
-      <c r="B31" s="28"/>
+      <c r="A31" s="32"/>
+      <c r="B31" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -2998,7 +3034,7 @@
   <dimension ref="A1:H55"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="23.7777777777778" style="8" customWidth="1"/>
+    <col min="1" max="1" width="23.7777777777778" style="11" customWidth="1"/>
     <col min="2" max="2" width="28.2222222222222" style="2" customWidth="1"/>
     <col min="3" max="3" width="11.2222222222222" style="2" customWidth="1"/>
     <col min="4" max="4" width="39" style="2" customWidth="1"/>
@@ -3009,1056 +3045,1056 @@
   </cols>
   <sheetData>
     <row r="1" ht="29" customHeight="1" spans="1:8">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
     </row>
     <row r="6" ht="31" customHeight="1" spans="1:8">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
     </row>
     <row r="9" ht="25" customHeight="1" spans="1:8">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="18" t="s">
         <v>130</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="20"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="17">
+      <c r="A11" s="21">
         <v>1</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="20" t="s">
         <v>133</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="22"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="17">
+      <c r="A12" s="21">
         <v>2</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="22" t="s">
         <v>136</v>
       </c>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="22"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="17">
+      <c r="A13" s="21">
         <v>3</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="17">
+      <c r="A14" s="21">
         <v>4</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="22"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="17">
+      <c r="A15" s="21">
         <v>5</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="17">
+      <c r="A16" s="21">
         <v>6</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="20" t="s">
         <v>143</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="17">
+      <c r="A17" s="21">
         <v>7</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="22" t="s">
         <v>146</v>
       </c>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="22"/>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="17">
+      <c r="A18" s="21">
         <v>8</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="20" t="s">
         <v>147</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="C18" s="22" t="s">
         <v>148</v>
       </c>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22"/>
+      <c r="H18" s="22"/>
     </row>
     <row r="19" spans="1:8">
-      <c r="A19" s="17">
+      <c r="A19" s="21">
         <v>9</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="20" t="s">
         <v>149</v>
       </c>
-      <c r="C19" s="18" t="s">
+      <c r="C19" s="22" t="s">
         <v>150</v>
       </c>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="22"/>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="17"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
+      <c r="A20" s="21"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="20"/>
     </row>
     <row r="21" ht="25" customHeight="1" spans="1:8">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="B21" s="19"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
+      <c r="B21" s="23"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="17"/>
     </row>
     <row r="22" spans="1:8">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="18" t="s">
         <v>151</v>
       </c>
-      <c r="B22" s="16" t="s">
+      <c r="B22" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="16" t="s">
+      <c r="C22" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="D22" s="16" t="s">
+      <c r="D22" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="E22" s="16" t="s">
+      <c r="E22" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="F22" s="16" t="s">
+      <c r="F22" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G22" s="16" t="s">
+      <c r="G22" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="H22" s="16" t="s">
+      <c r="H22" s="19" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="23" spans="1:8">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="20" t="s">
         <v>153</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="D23" s="20" t="s">
         <v>154</v>
       </c>
-      <c r="E23" s="5" t="s">
+      <c r="E23" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F23" s="5" t="s">
+      <c r="F23" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5" t="s">
+      <c r="G23" s="20"/>
+      <c r="H23" s="20" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="20" t="s">
         <v>156</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E24" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F24" s="5" t="s">
+      <c r="F24" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5" t="s">
+      <c r="G24" s="20"/>
+      <c r="H24" s="20" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="17" t="s">
+      <c r="A25" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5" t="s">
+      <c r="E25" s="20"/>
+      <c r="F25" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G25" s="5" t="s">
+      <c r="G25" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="H25" s="5" t="s">
+      <c r="H25" s="20" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="17" t="s">
+      <c r="A26" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="20" t="s">
         <v>161</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="D26" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5" t="s">
+      <c r="E26" s="20"/>
+      <c r="F26" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G26" s="20" t="s">
+      <c r="G26" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="H26" s="5" t="s">
+      <c r="H26" s="20" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="17" t="s">
+      <c r="A27" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="D27" s="20" t="s">
         <v>165</v>
       </c>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5" t="s">
+      <c r="E27" s="20"/>
+      <c r="F27" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G27" s="5" t="s">
+      <c r="G27" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="H27" s="5" t="s">
+      <c r="H27" s="20" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="28" ht="28.8" spans="1:8">
-      <c r="A28" s="17" t="s">
+      <c r="A28" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="20" t="s">
         <v>166</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="D28" s="20" t="s">
         <v>167</v>
       </c>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5" t="s">
+      <c r="E28" s="20"/>
+      <c r="F28" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G28" s="5"/>
-      <c r="H28" s="5" t="s">
+      <c r="G28" s="20"/>
+      <c r="H28" s="20" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="17" t="s">
+      <c r="A29" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="D29" s="20" t="s">
         <v>170</v>
       </c>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5" t="s">
+      <c r="E29" s="20"/>
+      <c r="F29" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G29" s="5"/>
-      <c r="H29" s="5" t="s">
+      <c r="G29" s="20"/>
+      <c r="H29" s="20" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="17" t="s">
+      <c r="A30" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="20" t="s">
         <v>172</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C30" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="D30" s="20" t="s">
         <v>173</v>
       </c>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5" t="s">
+      <c r="E30" s="20"/>
+      <c r="F30" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5" t="s">
+      <c r="G30" s="20"/>
+      <c r="H30" s="20" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="31" spans="1:8">
-      <c r="A31" s="17" t="s">
+      <c r="A31" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C31" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="D31" s="20" t="s">
         <v>176</v>
       </c>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5" t="s">
+      <c r="E31" s="20"/>
+      <c r="F31" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G31" s="5"/>
-      <c r="H31" s="5" t="s">
+      <c r="G31" s="20"/>
+      <c r="H31" s="20" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="32" spans="1:8">
-      <c r="A32" s="17" t="s">
+      <c r="A32" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="20" t="s">
         <v>177</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C32" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="D32" s="20" t="s">
         <v>178</v>
       </c>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5" t="s">
+      <c r="E32" s="20"/>
+      <c r="F32" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G32" s="5"/>
-      <c r="H32" s="5" t="s">
+      <c r="G32" s="20"/>
+      <c r="H32" s="20" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="33" spans="1:8">
-      <c r="A33" s="17" t="s">
+      <c r="A33" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="B33" s="20" t="s">
         <v>180</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C33" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="D33" s="20" t="s">
         <v>181</v>
       </c>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5" t="s">
+      <c r="E33" s="20"/>
+      <c r="F33" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G33" s="5"/>
-      <c r="H33" s="5" t="s">
+      <c r="G33" s="20"/>
+      <c r="H33" s="20" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="34" spans="1:8">
-      <c r="A34" s="17" t="s">
+      <c r="A34" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="20" t="s">
         <v>183</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="D34" s="20" t="s">
         <v>184</v>
       </c>
-      <c r="E34" s="5"/>
-      <c r="F34" s="5" t="s">
+      <c r="E34" s="20"/>
+      <c r="F34" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G34" s="5"/>
-      <c r="H34" s="5" t="s">
+      <c r="G34" s="20"/>
+      <c r="H34" s="20" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="35" ht="60" customHeight="1" spans="1:8">
-      <c r="A35" s="17" t="s">
+      <c r="A35" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="20" t="s">
         <v>186</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="C35" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="D35" s="21" t="s">
+      <c r="D35" s="25" t="s">
         <v>187</v>
       </c>
-      <c r="E35" s="31" t="s">
+      <c r="E35" s="35" t="s">
         <v>188</v>
       </c>
-      <c r="F35" s="5" t="s">
+      <c r="F35" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G35" s="5"/>
-      <c r="H35" s="5" t="s">
+      <c r="G35" s="20"/>
+      <c r="H35" s="20" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="36" spans="1:8">
-      <c r="A36" s="17" t="s">
+      <c r="A36" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="20" t="s">
         <v>190</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="C36" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="D36" s="20" t="s">
         <v>191</v>
       </c>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5" t="s">
+      <c r="E36" s="20"/>
+      <c r="F36" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G36" s="5"/>
-      <c r="H36" s="5" t="s">
+      <c r="G36" s="20"/>
+      <c r="H36" s="20" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="37" spans="1:8">
-      <c r="A37" s="17" t="s">
+      <c r="A37" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="20" t="s">
         <v>193</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C37" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="D37" s="5" t="s">
+      <c r="D37" s="20" t="s">
         <v>194</v>
       </c>
-      <c r="E37" s="5"/>
-      <c r="F37" s="5" t="s">
+      <c r="E37" s="20"/>
+      <c r="F37" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G37" s="5"/>
-      <c r="H37" s="5" t="s">
+      <c r="G37" s="20"/>
+      <c r="H37" s="20" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="38" spans="1:8">
-      <c r="A38" s="17" t="s">
+      <c r="A38" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="B38" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="C38" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="D38" s="20" t="s">
         <v>197</v>
       </c>
-      <c r="E38" s="5"/>
-      <c r="F38" s="5" t="s">
+      <c r="E38" s="20"/>
+      <c r="F38" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G38" s="5"/>
-      <c r="H38" s="5" t="s">
+      <c r="G38" s="20"/>
+      <c r="H38" s="20" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="39" spans="1:8">
-      <c r="A39" s="17" t="s">
+      <c r="A39" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="B39" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="C39" s="20" t="s">
         <v>200</v>
       </c>
-      <c r="D39" s="5" t="s">
+      <c r="D39" s="20" t="s">
         <v>201</v>
       </c>
-      <c r="E39" s="5"/>
-      <c r="F39" s="5" t="s">
+      <c r="E39" s="20"/>
+      <c r="F39" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G39" s="5"/>
-      <c r="H39" s="5" t="s">
+      <c r="G39" s="20"/>
+      <c r="H39" s="20" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="40" ht="28.8" spans="1:8">
-      <c r="A40" s="17" t="s">
+      <c r="A40" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="B40" s="20" t="s">
         <v>203</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="C40" s="20" t="s">
         <v>204</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="D40" s="20" t="s">
         <v>205</v>
       </c>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5" t="s">
+      <c r="E40" s="20"/>
+      <c r="F40" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5" t="s">
+      <c r="G40" s="20"/>
+      <c r="H40" s="20" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="41" ht="28.8" spans="1:8">
-      <c r="A41" s="17" t="s">
+      <c r="A41" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="B41" s="20" t="s">
         <v>207</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C41" s="20" t="s">
         <v>204</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="D41" s="20" t="s">
         <v>208</v>
       </c>
-      <c r="E41" s="5"/>
-      <c r="F41" s="5" t="s">
+      <c r="E41" s="20"/>
+      <c r="F41" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G41" s="5"/>
-      <c r="H41" s="5" t="s">
+      <c r="G41" s="20"/>
+      <c r="H41" s="20" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="42" ht="28.8" spans="1:8">
-      <c r="A42" s="17" t="s">
+      <c r="A42" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="B42" s="20" t="s">
         <v>209</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="C42" s="20" t="s">
         <v>204</v>
       </c>
-      <c r="D42" s="5" t="s">
+      <c r="D42" s="20" t="s">
         <v>210</v>
       </c>
-      <c r="E42" s="5"/>
-      <c r="F42" s="5" t="s">
+      <c r="E42" s="20"/>
+      <c r="F42" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G42" s="5"/>
-      <c r="H42" s="5" t="s">
+      <c r="G42" s="20"/>
+      <c r="H42" s="20" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="43" ht="28.8" spans="1:8">
-      <c r="A43" s="17" t="s">
+      <c r="A43" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="B43" s="20" t="s">
         <v>211</v>
       </c>
-      <c r="C43" s="5" t="s">
+      <c r="C43" s="20" t="s">
         <v>204</v>
       </c>
-      <c r="D43" s="5" t="s">
+      <c r="D43" s="20" t="s">
         <v>212</v>
       </c>
-      <c r="E43" s="5"/>
-      <c r="F43" s="5" t="s">
+      <c r="E43" s="20"/>
+      <c r="F43" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G43" s="5"/>
-      <c r="H43" s="5" t="s">
+      <c r="G43" s="20"/>
+      <c r="H43" s="20" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="44" spans="1:8">
-      <c r="A44" s="17" t="s">
+      <c r="A44" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="B44" s="20" t="s">
         <v>213</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="C44" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D44" s="5" t="s">
+      <c r="D44" s="20" t="s">
         <v>214</v>
       </c>
-      <c r="E44" s="5"/>
-      <c r="F44" s="5" t="s">
+      <c r="E44" s="20"/>
+      <c r="F44" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G44" s="5"/>
-      <c r="H44" s="5" t="s">
+      <c r="G44" s="20"/>
+      <c r="H44" s="20" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="45" spans="1:8">
-      <c r="A45" s="17" t="s">
+      <c r="A45" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="B45" s="20" t="s">
         <v>216</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="C45" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D45" s="5" t="s">
+      <c r="D45" s="20" t="s">
         <v>217</v>
       </c>
-      <c r="E45" s="5"/>
-      <c r="F45" s="5" t="s">
+      <c r="E45" s="20"/>
+      <c r="F45" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G45" s="5"/>
-      <c r="H45" s="5" t="s">
+      <c r="G45" s="20"/>
+      <c r="H45" s="20" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="46" spans="1:8">
-      <c r="A46" s="17" t="s">
+      <c r="A46" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B46" s="20" t="s">
         <v>218</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="C46" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D46" s="5" t="s">
+      <c r="D46" s="20" t="s">
         <v>219</v>
       </c>
-      <c r="E46" s="5"/>
-      <c r="F46" s="5" t="s">
+      <c r="E46" s="20"/>
+      <c r="F46" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G46" s="5"/>
-      <c r="H46" s="5" t="s">
+      <c r="G46" s="20"/>
+      <c r="H46" s="20" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="47" spans="1:8">
-      <c r="A47" s="17" t="s">
+      <c r="A47" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="B47" s="20" t="s">
         <v>221</v>
       </c>
-      <c r="C47" s="5" t="s">
+      <c r="C47" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D47" s="5" t="s">
+      <c r="D47" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="E47" s="5"/>
-      <c r="F47" s="5" t="s">
+      <c r="E47" s="20"/>
+      <c r="F47" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G47" s="5"/>
-      <c r="H47" s="5" t="s">
+      <c r="G47" s="20"/>
+      <c r="H47" s="20" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="48" spans="1:8">
-      <c r="A48" s="17" t="s">
+      <c r="A48" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="B48" s="5" t="s">
+      <c r="B48" s="20" t="s">
         <v>224</v>
       </c>
-      <c r="C48" s="5" t="s">
+      <c r="C48" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D48" s="5" t="s">
+      <c r="D48" s="20" t="s">
         <v>225</v>
       </c>
-      <c r="E48" s="5"/>
-      <c r="F48" s="5" t="s">
+      <c r="E48" s="20"/>
+      <c r="F48" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G48" s="5"/>
-      <c r="H48" s="5" t="s">
+      <c r="G48" s="20"/>
+      <c r="H48" s="20" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="49" spans="1:8">
-      <c r="A49" s="17" t="s">
+      <c r="A49" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B49" s="20" t="s">
         <v>226</v>
       </c>
-      <c r="C49" s="5" t="s">
+      <c r="C49" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D49" s="5" t="s">
+      <c r="D49" s="20" t="s">
         <v>227</v>
       </c>
-      <c r="E49" s="5"/>
-      <c r="F49" s="5" t="s">
+      <c r="E49" s="20"/>
+      <c r="F49" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G49" s="5"/>
-      <c r="H49" s="5" t="s">
+      <c r="G49" s="20"/>
+      <c r="H49" s="20" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="50" spans="1:8">
-      <c r="A50" s="17" t="s">
+      <c r="A50" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="B50" s="5" t="s">
+      <c r="B50" s="20" t="s">
         <v>228</v>
       </c>
-      <c r="C50" s="5" t="s">
+      <c r="C50" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D50" s="5" t="s">
+      <c r="D50" s="20" t="s">
         <v>229</v>
       </c>
-      <c r="E50" s="5"/>
-      <c r="F50" s="5" t="s">
+      <c r="E50" s="20"/>
+      <c r="F50" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G50" s="5"/>
-      <c r="H50" s="5" t="s">
+      <c r="G50" s="20"/>
+      <c r="H50" s="20" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="51" spans="1:8">
-      <c r="A51" s="17" t="s">
+      <c r="A51" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="B51" s="5" t="s">
+      <c r="B51" s="20" t="s">
         <v>230</v>
       </c>
-      <c r="C51" s="5" t="s">
+      <c r="C51" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D51" s="5" t="s">
+      <c r="D51" s="20" t="s">
         <v>231</v>
       </c>
-      <c r="E51" s="5"/>
-      <c r="F51" s="5" t="s">
+      <c r="E51" s="20"/>
+      <c r="F51" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G51" s="5"/>
-      <c r="H51" s="5" t="s">
+      <c r="G51" s="20"/>
+      <c r="H51" s="20" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="52" spans="1:8">
-      <c r="A52" s="17" t="s">
+      <c r="A52" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="B52" s="20" t="s">
         <v>233</v>
       </c>
-      <c r="C52" s="5" t="s">
+      <c r="C52" s="20" t="s">
         <v>234</v>
       </c>
-      <c r="D52" s="5" t="s">
+      <c r="D52" s="20" t="s">
         <v>235</v>
       </c>
-      <c r="E52" s="5"/>
-      <c r="F52" s="5" t="s">
+      <c r="E52" s="20"/>
+      <c r="F52" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G52" s="5"/>
-      <c r="H52" s="5" t="s">
+      <c r="G52" s="20"/>
+      <c r="H52" s="20" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="53" spans="1:8">
-      <c r="A53" s="17" t="s">
+      <c r="A53" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="B53" s="5" t="s">
+      <c r="B53" s="20" t="s">
         <v>237</v>
       </c>
-      <c r="C53" s="5" t="s">
+      <c r="C53" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D53" s="5" t="s">
+      <c r="D53" s="20" t="s">
         <v>238</v>
       </c>
-      <c r="E53" s="5"/>
-      <c r="F53" s="5" t="s">
+      <c r="E53" s="20"/>
+      <c r="F53" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G53" s="5"/>
-      <c r="H53" s="5" t="s">
+      <c r="G53" s="20"/>
+      <c r="H53" s="20" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="54" spans="1:8">
-      <c r="A54" s="17" t="s">
+      <c r="A54" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="B54" s="5" t="s">
+      <c r="B54" s="20" t="s">
         <v>240</v>
       </c>
-      <c r="C54" s="5" t="s">
+      <c r="C54" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D54" s="5" t="s">
+      <c r="D54" s="20" t="s">
         <v>241</v>
       </c>
-      <c r="E54" s="5"/>
-      <c r="F54" s="5" t="s">
+      <c r="E54" s="20"/>
+      <c r="F54" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G54" s="5"/>
-      <c r="H54" s="5" t="s">
+      <c r="G54" s="20"/>
+      <c r="H54" s="20" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="55" spans="1:8">
-      <c r="A55" s="17" t="s">
+      <c r="A55" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="B55" s="5" t="s">
+      <c r="B55" s="20" t="s">
         <v>242</v>
       </c>
-      <c r="C55" s="5" t="s">
+      <c r="C55" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D55" s="5" t="s">
+      <c r="D55" s="20" t="s">
         <v>243</v>
       </c>
-      <c r="E55" s="5"/>
-      <c r="F55" s="5" t="s">
+      <c r="E55" s="20"/>
+      <c r="F55" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G55" s="5"/>
-      <c r="H55" s="5" t="s">
+      <c r="G55" s="20"/>
+      <c r="H55" s="20" t="s">
         <v>239</v>
       </c>
     </row>
@@ -4142,7 +4178,7 @@
       <c r="H2" s="4" t="s">
         <v>252</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="8" t="s">
         <v>253</v>
       </c>
     </row>
@@ -4171,7 +4207,7 @@
       <c r="H3" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="9" t="s">
         <v>56</v>
       </c>
     </row>
@@ -4200,7 +4236,7 @@
       <c r="H4" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="9" t="s">
         <v>56</v>
       </c>
     </row>
@@ -4229,7 +4265,7 @@
       <c r="H5" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="9" t="s">
         <v>56</v>
       </c>
     </row>
@@ -4258,7 +4294,7 @@
       <c r="H6" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I6" s="9" t="s">
         <v>56</v>
       </c>
     </row>
@@ -4287,152 +4323,152 @@
       <c r="H7" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="8" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="7" t="s">
         <v>283</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="7" t="s">
         <v>284</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="7" t="s">
         <v>285</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="7" t="s">
         <v>286</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>260</v>
+      </c>
+      <c r="I8" s="10" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="9" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A9" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="B9" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>292</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="H9" s="7" t="s">
         <v>260</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I9" s="10" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="9" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
-      <c r="A9" s="5" t="s">
-        <v>288</v>
-      </c>
-      <c r="B9" s="5" t="s">
+    <row r="10" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A10" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>289</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>290</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>291</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>293</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>287</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>260</v>
-      </c>
-      <c r="I9" s="7" t="s">
+      <c r="D10" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="I10" s="10" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="10" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
-      <c r="A10" s="5" t="s">
-        <v>294</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>295</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>290</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>296</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>297</v>
-      </c>
-      <c r="F10" s="5" t="s">
+    <row r="11" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A11" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="H11" s="7" t="s">
         <v>298</v>
       </c>
-      <c r="G10" s="5" t="s">
-        <v>287</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>299</v>
-      </c>
-      <c r="I10" s="7" t="s">
+      <c r="I11" s="10" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="11" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
-      <c r="A11" s="5" t="s">
-        <v>300</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>301</v>
-      </c>
-      <c r="C11" s="5" t="s">
+    <row r="12" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
+      <c r="A12" s="6" t="s">
+        <v>304</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="C12" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>302</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>303</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>304</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>287</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>299</v>
-      </c>
-      <c r="I11" s="7" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="12" s="1" customFormat="1" ht="34" customHeight="1" spans="1:9">
-      <c r="A12" s="5" t="s">
-        <v>305</v>
-      </c>
-      <c r="B12" s="5" t="s">
+      <c r="D12" s="7" t="s">
         <v>306</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="D12" s="5" t="s">
+      <c r="E12" s="7" t="s">
         <v>307</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="F12" s="7" t="s">
         <v>308</v>
       </c>
-      <c r="F12" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>287</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>299</v>
-      </c>
-      <c r="I12" s="7" t="s">
+      <c r="G12" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="I12" s="10" t="s">
         <v>121</v>
       </c>
     </row>

</xml_diff>